<commit_message>
Update codebook procedure rater 1.xlsx
changed value of 1 cell bc of a mistake
</commit_message>
<xml_diff>
--- a/data/raw/metamethod review/codebook - rater 1/codebook procedure rater 1.xlsx
+++ b/data/raw/metamethod review/codebook - rater 1/codebook procedure rater 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Annika\Documents\01_STUDIUM\4. HTI\IGT Projekt\Codebook_new\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Annika\Documents\GitHub\IGT-project\data\raw\metamethod review\codebook - rater 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C47CCFE-2D76-438B-B8D9-E0ECBAF50A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1DAB8FA-7320-4B70-A012-E7E2B8382EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26475" yWindow="660" windowWidth="23925" windowHeight="19560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27165" yWindow="1350" windowWidth="23925" windowHeight="19560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1670,7 +1670,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1694,46 +1694,39 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2247,8 +2240,8 @@
       <c r="AD3" s="13" t="s">
         <v>417</v>
       </c>
-      <c r="AE3" s="14"/>
-      <c r="AF3" s="15"/>
+      <c r="AE3" s="5"/>
+      <c r="AF3" s="6"/>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
     </row>
@@ -2340,11 +2333,11 @@
       <c r="AC4" s="10">
         <v>100</v>
       </c>
-      <c r="AD4" s="16" t="s">
+      <c r="AD4" s="14" t="s">
         <v>383</v>
       </c>
-      <c r="AE4" s="14"/>
-      <c r="AF4" s="15"/>
+      <c r="AE4" s="5"/>
+      <c r="AF4" s="6"/>
       <c r="AG4" s="6"/>
       <c r="AH4" s="6"/>
     </row>
@@ -2440,8 +2433,8 @@
       <c r="AD5" s="11" t="s">
         <v>308</v>
       </c>
-      <c r="AE5" s="14"/>
-      <c r="AF5" s="15"/>
+      <c r="AE5" s="5"/>
+      <c r="AF5" s="6"/>
       <c r="AG5" s="6"/>
       <c r="AH5" s="6"/>
     </row>
@@ -2527,7 +2520,7 @@
       <c r="AA6" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="AB6" s="17" t="s">
+      <c r="AB6" s="15" t="s">
         <v>60</v>
       </c>
       <c r="AC6" s="10">
@@ -2536,8 +2529,8 @@
       <c r="AD6" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="AE6" s="14"/>
-      <c r="AF6" s="15"/>
+      <c r="AE6" s="5"/>
+      <c r="AF6" s="6"/>
       <c r="AG6" s="6"/>
       <c r="AH6" s="6"/>
     </row>
@@ -2632,8 +2625,8 @@
       <c r="AD7" s="11" t="s">
         <v>309</v>
       </c>
-      <c r="AE7" s="14"/>
-      <c r="AF7" s="15"/>
+      <c r="AE7" s="5"/>
+      <c r="AF7" s="6"/>
       <c r="AG7" s="6"/>
       <c r="AH7" s="6"/>
     </row>
@@ -2728,8 +2721,8 @@
       <c r="AD8" s="11" t="s">
         <v>310</v>
       </c>
-      <c r="AE8" s="14"/>
-      <c r="AF8" s="15"/>
+      <c r="AE8" s="5"/>
+      <c r="AF8" s="6"/>
       <c r="AG8" s="6"/>
       <c r="AH8" s="6"/>
     </row>
@@ -2821,11 +2814,11 @@
       <c r="AC9" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="AD9" s="18" t="s">
+      <c r="AD9" s="16" t="s">
         <v>441</v>
       </c>
-      <c r="AE9" s="14"/>
-      <c r="AF9" s="15"/>
+      <c r="AE9" s="5"/>
+      <c r="AF9" s="6"/>
       <c r="AG9" s="6"/>
       <c r="AH9" s="6"/>
     </row>
@@ -2857,10 +2850,10 @@
       <c r="I10" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="J10" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="K10" s="19" t="s">
+      <c r="J10" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="K10" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L10" s="10" t="s">
@@ -2899,16 +2892,16 @@
       <c r="W10" s="10">
         <v>10</v>
       </c>
-      <c r="X10" s="20">
+      <c r="X10" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y10" s="20">
+      <c r="Y10" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z10" s="20">
+      <c r="Z10" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA10" s="20">
+      <c r="AA10" s="18">
         <v>0.1</v>
       </c>
       <c r="AB10" s="10">
@@ -2917,11 +2910,11 @@
       <c r="AC10" s="10">
         <v>100</v>
       </c>
-      <c r="AD10" s="19" t="s">
+      <c r="AD10" s="17" t="s">
         <v>312</v>
       </c>
-      <c r="AE10" s="14"/>
-      <c r="AF10" s="15"/>
+      <c r="AE10" s="5"/>
+      <c r="AF10" s="6"/>
       <c r="AG10" s="6"/>
       <c r="AH10" s="6"/>
     </row>
@@ -2944,7 +2937,7 @@
       <c r="F11" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="21" t="s">
+      <c r="G11" s="19" t="s">
         <v>406</v>
       </c>
       <c r="H11" s="10" t="s">
@@ -2956,7 +2949,7 @@
       <c r="J11" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K11" s="19" t="s">
+      <c r="K11" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L11" s="10" t="s">
@@ -2995,16 +2988,16 @@
       <c r="W11" s="10">
         <v>10</v>
       </c>
-      <c r="X11" s="20">
+      <c r="X11" s="18">
         <v>0.25</v>
       </c>
-      <c r="Y11" s="20">
+      <c r="Y11" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z11" s="20">
+      <c r="Z11" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA11" s="20">
+      <c r="AA11" s="18">
         <v>0.1</v>
       </c>
       <c r="AB11" s="10">
@@ -3013,11 +3006,11 @@
       <c r="AC11" s="10">
         <v>120</v>
       </c>
-      <c r="AD11" s="22" t="s">
+      <c r="AD11" s="20" t="s">
         <v>407</v>
       </c>
-      <c r="AE11" s="14"/>
-      <c r="AF11" s="15"/>
+      <c r="AE11" s="5"/>
+      <c r="AF11" s="6"/>
       <c r="AG11" s="6"/>
       <c r="AH11" s="6"/>
     </row>
@@ -3040,7 +3033,7 @@
       <c r="F12" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G12" s="21" t="s">
+      <c r="G12" s="19" t="s">
         <v>313</v>
       </c>
       <c r="H12" s="10" t="s">
@@ -3073,10 +3066,10 @@
       <c r="Q12" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="R12" s="23" t="s">
+      <c r="R12" s="21" t="s">
         <v>398</v>
       </c>
-      <c r="S12" s="23" t="s">
+      <c r="S12" s="21" t="s">
         <v>398</v>
       </c>
       <c r="T12" s="10">
@@ -3094,13 +3087,13 @@
       <c r="X12" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="Y12" s="20">
+      <c r="Y12" s="18">
         <v>0.1</v>
       </c>
       <c r="Z12" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="AA12" s="20">
+      <c r="AA12" s="18">
         <v>0.1</v>
       </c>
       <c r="AB12" s="10">
@@ -3112,8 +3105,8 @@
       <c r="AD12" s="10" t="s">
         <v>392</v>
       </c>
-      <c r="AE12" s="14"/>
-      <c r="AF12" s="15"/>
+      <c r="AE12" s="5"/>
+      <c r="AF12" s="6"/>
       <c r="AG12" s="6"/>
       <c r="AH12" s="6"/>
     </row>
@@ -3137,7 +3130,7 @@
       <c r="F13" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G13" s="21" t="s">
+      <c r="G13" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H13" s="10" t="s">
@@ -3149,7 +3142,7 @@
       <c r="J13" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K13" s="19" t="s">
+      <c r="K13" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L13" s="10" t="s">
@@ -3209,8 +3202,8 @@
       <c r="AD13" s="10" t="s">
         <v>418</v>
       </c>
-      <c r="AE13" s="14"/>
-      <c r="AF13" s="15"/>
+      <c r="AE13" s="5"/>
+      <c r="AF13" s="6"/>
       <c r="AG13" s="6"/>
       <c r="AH13" s="6"/>
     </row>
@@ -3236,16 +3229,16 @@
       <c r="G14" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="17" t="s">
         <v>65</v>
       </c>
       <c r="I14" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="K14" s="19" t="s">
+      <c r="K14" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L14" s="10" t="s">
@@ -3284,16 +3277,16 @@
       <c r="W14" s="10">
         <v>10</v>
       </c>
-      <c r="X14" s="20">
+      <c r="X14" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y14" s="20">
+      <c r="Y14" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z14" s="20">
+      <c r="Z14" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA14" s="20">
+      <c r="AA14" s="18">
         <v>0.1</v>
       </c>
       <c r="AB14" s="10">
@@ -3302,11 +3295,11 @@
       <c r="AC14" s="10">
         <v>100</v>
       </c>
-      <c r="AD14" s="19" t="s">
+      <c r="AD14" s="17" t="s">
         <v>314</v>
       </c>
-      <c r="AE14" s="14"/>
-      <c r="AF14" s="15"/>
+      <c r="AE14" s="5"/>
+      <c r="AF14" s="6"/>
       <c r="AG14" s="6"/>
       <c r="AH14" s="6"/>
     </row>
@@ -3341,7 +3334,7 @@
       <c r="J15" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K15" s="19" t="s">
+      <c r="K15" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L15" s="10" t="s">
@@ -3380,16 +3373,16 @@
       <c r="W15" s="10">
         <v>10</v>
       </c>
-      <c r="X15" s="20">
+      <c r="X15" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y15" s="20">
+      <c r="Y15" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z15" s="20">
+      <c r="Z15" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA15" s="20">
+      <c r="AA15" s="18">
         <v>0.1</v>
       </c>
       <c r="AB15" s="10" t="s">
@@ -3398,11 +3391,11 @@
       <c r="AC15" s="10">
         <v>100</v>
       </c>
-      <c r="AD15" s="22" t="s">
+      <c r="AD15" s="20" t="s">
         <v>400</v>
       </c>
-      <c r="AE15" s="14"/>
-      <c r="AF15" s="15"/>
+      <c r="AE15" s="5"/>
+      <c r="AF15" s="6"/>
       <c r="AG15" s="6"/>
       <c r="AH15" s="6"/>
     </row>
@@ -3428,13 +3421,13 @@
       <c r="G16" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I16" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="J16" s="19" t="s">
+      <c r="I16" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J16" s="17" t="s">
         <v>61</v>
       </c>
       <c r="K16" s="10" t="s">
@@ -3476,16 +3469,16 @@
       <c r="W16" s="10">
         <v>10</v>
       </c>
-      <c r="X16" s="20">
+      <c r="X16" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y16" s="20">
+      <c r="Y16" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z16" s="20">
+      <c r="Z16" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA16" s="20">
+      <c r="AA16" s="18">
         <v>0.1</v>
       </c>
       <c r="AB16" s="10">
@@ -3494,11 +3487,11 @@
       <c r="AC16" s="10">
         <v>100</v>
       </c>
-      <c r="AD16" s="19" t="s">
+      <c r="AD16" s="17" t="s">
         <v>318</v>
       </c>
-      <c r="AE16" s="14"/>
-      <c r="AF16" s="15"/>
+      <c r="AE16" s="5"/>
+      <c r="AF16" s="6"/>
       <c r="AG16" s="6"/>
       <c r="AH16" s="6"/>
     </row>
@@ -3524,19 +3517,19 @@
       <c r="G17" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I17" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="J17" s="19" t="s">
+      <c r="I17" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J17" s="17" t="s">
         <v>61</v>
       </c>
       <c r="K17" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L17" s="19" t="s">
+      <c r="L17" s="17" t="s">
         <v>61</v>
       </c>
       <c r="M17" s="10" t="s">
@@ -3590,11 +3583,11 @@
       <c r="AC17" s="10">
         <v>100</v>
       </c>
-      <c r="AD17" s="19" t="s">
+      <c r="AD17" s="17" t="s">
         <v>317</v>
       </c>
-      <c r="AE17" s="14"/>
-      <c r="AF17" s="15"/>
+      <c r="AE17" s="5"/>
+      <c r="AF17" s="6"/>
       <c r="AG17" s="6"/>
       <c r="AH17" s="6"/>
     </row>
@@ -3653,7 +3646,7 @@
       <c r="R18" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="S18" s="19" t="s">
+      <c r="S18" s="17" t="s">
         <v>61</v>
       </c>
       <c r="T18" s="10" t="s">
@@ -3686,11 +3679,11 @@
       <c r="AC18" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="AD18" s="19" t="s">
+      <c r="AD18" s="17" t="s">
         <v>317</v>
       </c>
-      <c r="AE18" s="14"/>
-      <c r="AF18" s="15"/>
+      <c r="AE18" s="5"/>
+      <c r="AF18" s="6"/>
       <c r="AG18" s="6"/>
       <c r="AH18" s="6"/>
     </row>
@@ -3716,13 +3709,13 @@
       <c r="G19" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="H19" s="19" t="s">
+      <c r="H19" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I19" s="19" t="s">
+      <c r="I19" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="J19" s="19" t="s">
+      <c r="J19" s="17" t="s">
         <v>67</v>
       </c>
       <c r="K19" s="10" t="s">
@@ -3764,16 +3757,16 @@
       <c r="W19" s="10">
         <v>10</v>
       </c>
-      <c r="X19" s="20">
+      <c r="X19" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y19" s="20">
+      <c r="Y19" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z19" s="20">
+      <c r="Z19" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA19" s="20">
+      <c r="AA19" s="18">
         <v>0.1</v>
       </c>
       <c r="AB19" s="10">
@@ -3785,8 +3778,8 @@
       <c r="AD19" s="10" t="s">
         <v>438</v>
       </c>
-      <c r="AE19" s="14"/>
-      <c r="AF19" s="15"/>
+      <c r="AE19" s="5"/>
+      <c r="AF19" s="6"/>
       <c r="AG19" s="6"/>
       <c r="AH19" s="6"/>
     </row>
@@ -3881,8 +3874,8 @@
       <c r="AD20" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="AE20" s="14"/>
-      <c r="AF20" s="15"/>
+      <c r="AE20" s="5"/>
+      <c r="AF20" s="6"/>
       <c r="AG20" s="6"/>
       <c r="AH20" s="6"/>
     </row>
@@ -3977,8 +3970,8 @@
       <c r="AD21" s="13" t="s">
         <v>419</v>
       </c>
-      <c r="AE21" s="14"/>
-      <c r="AF21" s="15"/>
+      <c r="AE21" s="5"/>
+      <c r="AF21" s="6"/>
       <c r="AG21" s="6"/>
       <c r="AH21" s="6"/>
     </row>
@@ -4013,7 +4006,7 @@
       <c r="J22" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="K22" s="19" t="s">
+      <c r="K22" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L22" s="11" t="s">
@@ -4034,10 +4027,10 @@
       <c r="Q22" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="R22" s="23" t="s">
+      <c r="R22" s="21" t="s">
         <v>398</v>
       </c>
-      <c r="S22" s="23" t="s">
+      <c r="S22" s="21" t="s">
         <v>398</v>
       </c>
       <c r="T22" s="10">
@@ -4055,13 +4048,13 @@
       <c r="X22" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="Y22" s="20">
+      <c r="Y22" s="18">
         <v>0.1</v>
       </c>
       <c r="Z22" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="AA22" s="20">
+      <c r="AA22" s="18">
         <v>0.1</v>
       </c>
       <c r="AB22" s="10">
@@ -4070,11 +4063,11 @@
       <c r="AC22" s="10">
         <v>100</v>
       </c>
-      <c r="AD22" s="22" t="s">
+      <c r="AD22" s="20" t="s">
         <v>420</v>
       </c>
-      <c r="AE22" s="14"/>
-      <c r="AF22" s="15"/>
+      <c r="AE22" s="5"/>
+      <c r="AF22" s="6"/>
       <c r="AG22" s="6"/>
       <c r="AH22" s="6"/>
     </row>
@@ -4100,13 +4093,13 @@
       <c r="G23" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I23" s="19" t="s">
+      <c r="I23" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="J23" s="19" t="s">
+      <c r="J23" s="17" t="s">
         <v>67</v>
       </c>
       <c r="K23" s="10" t="s">
@@ -4148,16 +4141,16 @@
       <c r="W23" s="10">
         <v>10</v>
       </c>
-      <c r="X23" s="20">
+      <c r="X23" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y23" s="20">
+      <c r="Y23" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z23" s="20">
+      <c r="Z23" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA23" s="20">
+      <c r="AA23" s="18">
         <v>0.1</v>
       </c>
       <c r="AB23" s="10">
@@ -4166,11 +4159,11 @@
       <c r="AC23" s="10">
         <v>100</v>
       </c>
-      <c r="AD23" s="19" t="s">
+      <c r="AD23" s="17" t="s">
         <v>320</v>
       </c>
-      <c r="AE23" s="14"/>
-      <c r="AF23" s="15"/>
+      <c r="AE23" s="5"/>
+      <c r="AF23" s="6"/>
       <c r="AG23" s="6"/>
       <c r="AH23" s="6"/>
     </row>
@@ -4196,13 +4189,13 @@
       <c r="G24" s="12" t="s">
         <v>408</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="H24" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="I24" s="19" t="s">
+      <c r="I24" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="J24" s="19" t="s">
+      <c r="J24" s="17" t="s">
         <v>71</v>
       </c>
       <c r="K24" s="10" t="s">
@@ -4244,16 +4237,16 @@
       <c r="W24" s="10">
         <v>10</v>
       </c>
-      <c r="X24" s="20">
+      <c r="X24" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y24" s="20">
+      <c r="Y24" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z24" s="20">
+      <c r="Z24" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA24" s="20">
+      <c r="AA24" s="18">
         <v>0.1</v>
       </c>
       <c r="AB24" s="10">
@@ -4262,11 +4255,11 @@
       <c r="AC24" s="10">
         <v>100</v>
       </c>
-      <c r="AD24" s="19" t="s">
+      <c r="AD24" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="AE24" s="14"/>
-      <c r="AF24" s="15"/>
+      <c r="AE24" s="5"/>
+      <c r="AF24" s="6"/>
       <c r="AG24" s="6"/>
       <c r="AH24" s="6"/>
     </row>
@@ -4355,14 +4348,14 @@
       <c r="AB25" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="AC25" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD25" s="19" t="s">
+      <c r="AC25" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="AD25" s="17" t="s">
         <v>322</v>
       </c>
-      <c r="AE25" s="14"/>
-      <c r="AF25" s="15"/>
+      <c r="AE25" s="5"/>
+      <c r="AF25" s="6"/>
       <c r="AG25" s="6"/>
       <c r="AH25" s="6"/>
     </row>
@@ -4389,7 +4382,7 @@
       <c r="G26" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H26" s="19" t="s">
+      <c r="H26" s="17" t="s">
         <v>65</v>
       </c>
       <c r="I26" s="10" t="s">
@@ -4398,10 +4391,10 @@
       <c r="J26" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K26" s="19" t="s">
+      <c r="K26" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="L26" s="19" t="s">
+      <c r="L26" s="17" t="s">
         <v>61</v>
       </c>
       <c r="M26" s="10" t="s">
@@ -4455,11 +4448,11 @@
       <c r="AC26" s="10">
         <v>100</v>
       </c>
-      <c r="AD26" s="24" t="s">
+      <c r="AD26" s="22" t="s">
         <v>384</v>
       </c>
-      <c r="AE26" s="14"/>
-      <c r="AF26" s="15"/>
+      <c r="AE26" s="5"/>
+      <c r="AF26" s="6"/>
       <c r="AG26" s="6"/>
       <c r="AH26" s="6"/>
     </row>
@@ -4494,7 +4487,7 @@
       <c r="J27" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K27" s="19" t="s">
+      <c r="K27" s="17" t="s">
         <v>319</v>
       </c>
       <c r="L27" s="11" t="s">
@@ -4509,16 +4502,16 @@
       <c r="O27" s="10">
         <v>100</v>
       </c>
-      <c r="P27" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q27" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="R27" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="S27" s="19" t="s">
+      <c r="P27" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q27" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="R27" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="S27" s="17" t="s">
         <v>61</v>
       </c>
       <c r="T27" s="10" t="s">
@@ -4551,11 +4544,11 @@
       <c r="AC27" s="10">
         <v>100</v>
       </c>
-      <c r="AD27" s="22" t="s">
+      <c r="AD27" s="20" t="s">
         <v>323</v>
       </c>
-      <c r="AE27" s="14"/>
-      <c r="AF27" s="15"/>
+      <c r="AE27" s="5"/>
+      <c r="AF27" s="6"/>
       <c r="AG27" s="6"/>
       <c r="AH27" s="6"/>
     </row>
@@ -4581,13 +4574,13 @@
       <c r="G28" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H28" s="19" t="s">
+      <c r="H28" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I28" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="J28" s="19" t="s">
+      <c r="I28" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J28" s="17" t="s">
         <v>67</v>
       </c>
       <c r="K28" s="10" t="s">
@@ -4629,16 +4622,16 @@
       <c r="W28" s="10">
         <v>10</v>
       </c>
-      <c r="X28" s="20">
+      <c r="X28" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y28" s="20">
+      <c r="Y28" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z28" s="20">
+      <c r="Z28" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA28" s="20">
+      <c r="AA28" s="18">
         <v>0.1</v>
       </c>
       <c r="AB28" s="10" t="s">
@@ -4647,11 +4640,11 @@
       <c r="AC28" s="10">
         <v>100</v>
       </c>
-      <c r="AD28" s="19" t="s">
+      <c r="AD28" s="17" t="s">
         <v>324</v>
       </c>
-      <c r="AE28" s="14"/>
-      <c r="AF28" s="15"/>
+      <c r="AE28" s="5"/>
+      <c r="AF28" s="6"/>
       <c r="AG28" s="6"/>
       <c r="AH28" s="6"/>
     </row>
@@ -4743,11 +4736,11 @@
       <c r="AC29" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="AD29" s="19" t="s">
+      <c r="AD29" s="17" t="s">
         <v>294</v>
       </c>
-      <c r="AE29" s="14"/>
-      <c r="AF29" s="15"/>
+      <c r="AE29" s="5"/>
+      <c r="AF29" s="6"/>
       <c r="AG29" s="6"/>
       <c r="AH29" s="6"/>
     </row>
@@ -4773,7 +4766,7 @@
       <c r="G30" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="H30" s="17" t="s">
         <v>65</v>
       </c>
       <c r="I30" s="10" t="s">
@@ -4839,11 +4832,11 @@
       <c r="AC30" s="10">
         <v>100</v>
       </c>
-      <c r="AD30" s="19" t="s">
+      <c r="AD30" s="17" t="s">
         <v>325</v>
       </c>
-      <c r="AE30" s="14"/>
-      <c r="AF30" s="15"/>
+      <c r="AE30" s="5"/>
+      <c r="AF30" s="6"/>
       <c r="AG30" s="6"/>
       <c r="AH30" s="6"/>
     </row>
@@ -4872,10 +4865,10 @@
       <c r="H31" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I31" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="J31" s="19" t="s">
+      <c r="I31" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J31" s="17" t="s">
         <v>61</v>
       </c>
       <c r="K31" s="10" t="s">
@@ -4917,16 +4910,16 @@
       <c r="W31" s="10">
         <v>10</v>
       </c>
-      <c r="X31" s="20">
+      <c r="X31" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y31" s="20">
+      <c r="Y31" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z31" s="20">
+      <c r="Z31" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA31" s="20">
+      <c r="AA31" s="18">
         <v>0.1</v>
       </c>
       <c r="AB31" s="10" t="s">
@@ -4935,11 +4928,11 @@
       <c r="AC31" s="10">
         <v>100</v>
       </c>
-      <c r="AD31" s="19" t="s">
+      <c r="AD31" s="17" t="s">
         <v>385</v>
       </c>
-      <c r="AE31" s="14"/>
-      <c r="AF31" s="15"/>
+      <c r="AE31" s="5"/>
+      <c r="AF31" s="6"/>
       <c r="AG31" s="6"/>
       <c r="AH31" s="6"/>
     </row>
@@ -4965,10 +4958,10 @@
       <c r="G32" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H32" s="19" t="s">
+      <c r="H32" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I32" s="19" t="s">
+      <c r="I32" s="17" t="s">
         <v>66</v>
       </c>
       <c r="J32" s="10" t="s">
@@ -5013,16 +5006,16 @@
       <c r="W32" s="10">
         <v>10</v>
       </c>
-      <c r="X32" s="20">
+      <c r="X32" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y32" s="20">
+      <c r="Y32" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z32" s="20">
+      <c r="Z32" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA32" s="20">
+      <c r="AA32" s="18">
         <v>0.1</v>
       </c>
       <c r="AB32" s="10">
@@ -5031,11 +5024,11 @@
       <c r="AC32" s="10">
         <v>100</v>
       </c>
-      <c r="AD32" s="19" t="s">
+      <c r="AD32" s="17" t="s">
         <v>326</v>
       </c>
-      <c r="AE32" s="14"/>
-      <c r="AF32" s="15"/>
+      <c r="AE32" s="5"/>
+      <c r="AF32" s="6"/>
       <c r="AG32" s="6"/>
       <c r="AH32" s="6"/>
     </row>
@@ -5064,13 +5057,13 @@
       <c r="H33" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I33" s="19" t="s">
+      <c r="I33" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="J33" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="K33" s="19" t="s">
+      <c r="J33" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="K33" s="17" t="s">
         <v>319</v>
       </c>
       <c r="L33" s="11" t="s">
@@ -5109,16 +5102,16 @@
       <c r="W33" s="10">
         <v>10</v>
       </c>
-      <c r="X33" s="20">
+      <c r="X33" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y33" s="20">
+      <c r="Y33" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z33" s="20">
+      <c r="Z33" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA33" s="20">
+      <c r="AA33" s="18">
         <v>0.1</v>
       </c>
       <c r="AB33" s="10">
@@ -5127,11 +5120,11 @@
       <c r="AC33" s="10">
         <v>135</v>
       </c>
-      <c r="AD33" s="19" t="s">
+      <c r="AD33" s="17" t="s">
         <v>327</v>
       </c>
-      <c r="AE33" s="14"/>
-      <c r="AF33" s="15"/>
+      <c r="AE33" s="5"/>
+      <c r="AF33" s="6"/>
       <c r="AG33" s="6"/>
       <c r="AH33" s="6"/>
     </row>
@@ -5226,8 +5219,8 @@
       <c r="AD34" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="AE34" s="14"/>
-      <c r="AF34" s="15"/>
+      <c r="AE34" s="5"/>
+      <c r="AF34" s="6"/>
       <c r="AG34" s="6"/>
       <c r="AH34" s="6"/>
     </row>
@@ -5256,16 +5249,16 @@
       <c r="H35" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="I35" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="J35" s="19" t="s">
+      <c r="I35" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J35" s="17" t="s">
         <v>61</v>
       </c>
       <c r="K35" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L35" s="19" t="s">
+      <c r="L35" s="17" t="s">
         <v>61</v>
       </c>
       <c r="M35" s="10" t="s">
@@ -5319,11 +5312,11 @@
       <c r="AC35" s="10">
         <v>100</v>
       </c>
-      <c r="AD35" s="19" t="s">
+      <c r="AD35" s="17" t="s">
         <v>328</v>
       </c>
-      <c r="AE35" s="14"/>
-      <c r="AF35" s="15"/>
+      <c r="AE35" s="5"/>
+      <c r="AF35" s="6"/>
       <c r="AG35" s="6"/>
       <c r="AH35" s="6"/>
     </row>
@@ -5350,19 +5343,19 @@
       <c r="G36" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H36" s="19" t="s">
+      <c r="H36" s="17" t="s">
         <v>65</v>
       </c>
       <c r="I36" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="J36" s="19" t="s">
+      <c r="J36" s="17" t="s">
         <v>61</v>
       </c>
       <c r="K36" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L36" s="19" t="s">
+      <c r="L36" s="17" t="s">
         <v>61</v>
       </c>
       <c r="M36" s="10" t="s">
@@ -5416,11 +5409,11 @@
       <c r="AC36" s="10">
         <v>100</v>
       </c>
-      <c r="AD36" s="19" t="s">
+      <c r="AD36" s="17" t="s">
         <v>329</v>
       </c>
-      <c r="AE36" s="14"/>
-      <c r="AF36" s="15"/>
+      <c r="AE36" s="5"/>
+      <c r="AF36" s="6"/>
       <c r="AG36" s="6"/>
       <c r="AH36" s="6"/>
     </row>
@@ -5446,13 +5439,13 @@
       <c r="G37" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="H37" s="19" t="s">
+      <c r="H37" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I37" s="19" t="s">
+      <c r="I37" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="J37" s="19" t="s">
+      <c r="J37" s="17" t="s">
         <v>67</v>
       </c>
       <c r="K37" s="10" t="s">
@@ -5494,16 +5487,16 @@
       <c r="W37" s="10">
         <v>10</v>
       </c>
-      <c r="X37" s="20">
+      <c r="X37" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y37" s="20">
+      <c r="Y37" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z37" s="20">
+      <c r="Z37" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA37" s="20">
+      <c r="AA37" s="18">
         <v>0.1</v>
       </c>
       <c r="AB37" s="10">
@@ -5512,11 +5505,11 @@
       <c r="AC37" s="10">
         <v>100</v>
       </c>
-      <c r="AD37" s="22" t="s">
+      <c r="AD37" s="20" t="s">
         <v>416</v>
       </c>
-      <c r="AE37" s="14"/>
-      <c r="AF37" s="15"/>
+      <c r="AE37" s="5"/>
+      <c r="AF37" s="6"/>
       <c r="AG37" s="6"/>
       <c r="AH37" s="6"/>
     </row>
@@ -5543,7 +5536,7 @@
       <c r="G38" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H38" s="19" t="s">
+      <c r="H38" s="17" t="s">
         <v>65</v>
       </c>
       <c r="I38" s="10" t="s">
@@ -5555,7 +5548,7 @@
       <c r="K38" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L38" s="19" t="s">
+      <c r="L38" s="17" t="s">
         <v>61</v>
       </c>
       <c r="M38" s="10" t="s">
@@ -5609,11 +5602,11 @@
       <c r="AC38" s="10">
         <v>100</v>
       </c>
-      <c r="AD38" s="19" t="s">
+      <c r="AD38" s="17" t="s">
         <v>330</v>
       </c>
-      <c r="AE38" s="14"/>
-      <c r="AF38" s="15"/>
+      <c r="AE38" s="5"/>
+      <c r="AF38" s="6"/>
       <c r="AG38" s="6"/>
       <c r="AH38" s="6"/>
     </row>
@@ -5705,11 +5698,11 @@
       <c r="AC39" s="10">
         <v>100</v>
       </c>
-      <c r="AD39" s="19" t="s">
+      <c r="AD39" s="17" t="s">
         <v>331</v>
       </c>
-      <c r="AE39" s="14"/>
-      <c r="AF39" s="15"/>
+      <c r="AE39" s="5"/>
+      <c r="AF39" s="6"/>
       <c r="AG39" s="6"/>
       <c r="AH39" s="6"/>
     </row>
@@ -5736,13 +5729,13 @@
       <c r="G40" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H40" s="19" t="s">
+      <c r="H40" s="17" t="s">
         <v>65</v>
       </c>
       <c r="I40" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="J40" s="19" t="s">
+      <c r="J40" s="17" t="s">
         <v>61</v>
       </c>
       <c r="K40" s="10" t="s">
@@ -5805,8 +5798,8 @@
       <c r="AD40" s="13" t="s">
         <v>421</v>
       </c>
-      <c r="AE40" s="14"/>
-      <c r="AF40" s="15"/>
+      <c r="AE40" s="5"/>
+      <c r="AF40" s="6"/>
       <c r="AG40" s="6"/>
       <c r="AH40" s="6"/>
     </row>
@@ -5832,16 +5825,16 @@
       <c r="G41" s="12" t="s">
         <v>311</v>
       </c>
-      <c r="H41" s="19" t="s">
+      <c r="H41" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I41" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="J41" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="K41" s="19" t="s">
+      <c r="I41" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J41" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="K41" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L41" s="11" t="s">
@@ -5901,8 +5894,8 @@
       <c r="AD41" s="13" t="s">
         <v>422</v>
       </c>
-      <c r="AE41" s="14"/>
-      <c r="AF41" s="15"/>
+      <c r="AE41" s="5"/>
+      <c r="AF41" s="6"/>
       <c r="AG41" s="6"/>
       <c r="AH41" s="6"/>
     </row>
@@ -5928,13 +5921,13 @@
       <c r="G42" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H42" s="19" t="s">
+      <c r="H42" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="I42" s="19" t="s">
+      <c r="I42" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="J42" s="19" t="s">
+      <c r="J42" s="17" t="s">
         <v>71</v>
       </c>
       <c r="K42" s="10" t="s">
@@ -5976,16 +5969,16 @@
       <c r="W42" s="10">
         <v>10</v>
       </c>
-      <c r="X42" s="20">
+      <c r="X42" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y42" s="20">
+      <c r="Y42" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z42" s="20">
+      <c r="Z42" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA42" s="20">
+      <c r="AA42" s="18">
         <v>0.1</v>
       </c>
       <c r="AB42" s="10">
@@ -5994,11 +5987,11 @@
       <c r="AC42" s="10">
         <v>100</v>
       </c>
-      <c r="AD42" s="19" t="s">
+      <c r="AD42" s="17" t="s">
         <v>332</v>
       </c>
-      <c r="AE42" s="14"/>
-      <c r="AF42" s="15"/>
+      <c r="AE42" s="5"/>
+      <c r="AF42" s="6"/>
       <c r="AG42" s="6"/>
       <c r="AH42" s="6"/>
     </row>
@@ -6021,7 +6014,7 @@
       <c r="F43" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G43" s="21" t="s">
+      <c r="G43" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H43" s="10" t="s">
@@ -6072,16 +6065,16 @@
       <c r="W43" s="10">
         <v>10</v>
       </c>
-      <c r="X43" s="20">
+      <c r="X43" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y43" s="20">
+      <c r="Y43" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z43" s="20">
+      <c r="Z43" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA43" s="20">
+      <c r="AA43" s="18">
         <v>0.1</v>
       </c>
       <c r="AB43" s="10" t="s">
@@ -6093,8 +6086,8 @@
       <c r="AD43" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="AE43" s="14"/>
-      <c r="AF43" s="15"/>
+      <c r="AE43" s="5"/>
+      <c r="AF43" s="6"/>
       <c r="AG43" s="6"/>
       <c r="AH43" s="6"/>
     </row>
@@ -6117,7 +6110,7 @@
       <c r="F44" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G44" s="21" t="s">
+      <c r="G44" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H44" s="10" t="s">
@@ -6132,7 +6125,7 @@
       <c r="K44" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L44" s="25" t="s">
+      <c r="L44" s="23" t="s">
         <v>61</v>
       </c>
       <c r="M44" s="10" t="s">
@@ -6189,8 +6182,8 @@
       <c r="AD44" s="10" t="s">
         <v>334</v>
       </c>
-      <c r="AE44" s="14"/>
-      <c r="AF44" s="15"/>
+      <c r="AE44" s="5"/>
+      <c r="AF44" s="6"/>
       <c r="AG44" s="6"/>
       <c r="AH44" s="6"/>
     </row>
@@ -6213,7 +6206,7 @@
       <c r="F45" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G45" s="21" t="s">
+      <c r="G45" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H45" s="10" t="s">
@@ -6228,7 +6221,7 @@
       <c r="K45" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L45" s="25" t="s">
+      <c r="L45" s="23" t="s">
         <v>61</v>
       </c>
       <c r="M45" s="10" t="s">
@@ -6282,11 +6275,11 @@
       <c r="AC45" s="10">
         <v>100</v>
       </c>
-      <c r="AD45" s="25" t="s">
+      <c r="AD45" s="23" t="s">
         <v>335</v>
       </c>
-      <c r="AE45" s="14"/>
-      <c r="AF45" s="15"/>
+      <c r="AE45" s="5"/>
+      <c r="AF45" s="6"/>
       <c r="AG45" s="6"/>
       <c r="AH45" s="6"/>
     </row>
@@ -6309,7 +6302,7 @@
       <c r="F46" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G46" s="21" t="s">
+      <c r="G46" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H46" s="10" t="s">
@@ -6381,8 +6374,8 @@
       <c r="AD46" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="AE46" s="14"/>
-      <c r="AF46" s="15"/>
+      <c r="AE46" s="5"/>
+      <c r="AF46" s="6"/>
       <c r="AG46" s="6"/>
       <c r="AH46" s="6"/>
     </row>
@@ -6405,7 +6398,7 @@
       <c r="F47" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G47" s="21" t="s">
+      <c r="G47" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H47" s="10" t="s">
@@ -6420,7 +6413,7 @@
       <c r="K47" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L47" s="25" t="s">
+      <c r="L47" s="23" t="s">
         <v>61</v>
       </c>
       <c r="M47" s="10" t="s">
@@ -6477,8 +6470,8 @@
       <c r="AD47" s="10" t="s">
         <v>439</v>
       </c>
-      <c r="AE47" s="14"/>
-      <c r="AF47" s="15"/>
+      <c r="AE47" s="5"/>
+      <c r="AF47" s="6"/>
       <c r="AG47" s="6"/>
       <c r="AH47" s="6"/>
     </row>
@@ -6501,7 +6494,7 @@
       <c r="F48" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G48" s="21" t="s">
+      <c r="G48" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H48" s="10" t="s">
@@ -6516,7 +6509,7 @@
       <c r="K48" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L48" s="25" t="s">
+      <c r="L48" s="23" t="s">
         <v>61</v>
       </c>
       <c r="M48" s="10" t="s">
@@ -6573,8 +6566,8 @@
       <c r="AD48" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="AE48" s="14"/>
-      <c r="AF48" s="15"/>
+      <c r="AE48" s="5"/>
+      <c r="AF48" s="6"/>
       <c r="AG48" s="6"/>
       <c r="AH48" s="6"/>
     </row>
@@ -6598,7 +6591,7 @@
       <c r="F49" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G49" s="21" t="s">
+      <c r="G49" s="19" t="s">
         <v>338</v>
       </c>
       <c r="H49" s="10" t="s">
@@ -6649,16 +6642,16 @@
       <c r="W49" s="10">
         <v>20</v>
       </c>
-      <c r="X49" s="20">
+      <c r="X49" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y49" s="20">
+      <c r="Y49" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z49" s="20">
+      <c r="Z49" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA49" s="20">
+      <c r="AA49" s="18">
         <v>0.1</v>
       </c>
       <c r="AB49" s="10">
@@ -6670,8 +6663,8 @@
       <c r="AD49" s="10" t="s">
         <v>402</v>
       </c>
-      <c r="AE49" s="14"/>
-      <c r="AF49" s="15"/>
+      <c r="AE49" s="5"/>
+      <c r="AF49" s="6"/>
       <c r="AG49" s="6"/>
       <c r="AH49" s="6"/>
     </row>
@@ -6694,7 +6687,7 @@
       <c r="F50" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G50" s="21" t="s">
+      <c r="G50" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H50" s="10" t="s">
@@ -6766,8 +6759,8 @@
       <c r="AD50" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="AE50" s="14"/>
-      <c r="AF50" s="15"/>
+      <c r="AE50" s="5"/>
+      <c r="AF50" s="6"/>
       <c r="AG50" s="6"/>
       <c r="AH50" s="6"/>
     </row>
@@ -6790,7 +6783,7 @@
       <c r="F51" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G51" s="21" t="s">
+      <c r="G51" s="19" t="s">
         <v>311</v>
       </c>
       <c r="H51" s="10" t="s">
@@ -6802,7 +6795,7 @@
       <c r="J51" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K51" s="19" t="s">
+      <c r="K51" s="17" t="s">
         <v>319</v>
       </c>
       <c r="L51" s="11" t="s">
@@ -6859,11 +6852,11 @@
       <c r="AC51" s="10">
         <v>100</v>
       </c>
-      <c r="AD51" s="26" t="s">
+      <c r="AD51" s="24" t="s">
         <v>340</v>
       </c>
-      <c r="AE51" s="14"/>
-      <c r="AF51" s="15"/>
+      <c r="AE51" s="5"/>
+      <c r="AF51" s="6"/>
       <c r="AG51" s="6"/>
       <c r="AH51" s="6"/>
     </row>
@@ -6886,7 +6879,7 @@
       <c r="F52" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G52" s="21" t="s">
+      <c r="G52" s="19" t="s">
         <v>64</v>
       </c>
       <c r="H52" s="10" t="s">
@@ -6937,16 +6930,16 @@
       <c r="W52" s="10">
         <v>10</v>
       </c>
-      <c r="X52" s="20">
+      <c r="X52" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y52" s="20">
+      <c r="Y52" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z52" s="20">
+      <c r="Z52" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA52" s="20">
+      <c r="AA52" s="18">
         <v>0.1</v>
       </c>
       <c r="AB52" s="10">
@@ -6958,8 +6951,8 @@
       <c r="AD52" s="10" t="s">
         <v>386</v>
       </c>
-      <c r="AE52" s="14"/>
-      <c r="AF52" s="15"/>
+      <c r="AE52" s="5"/>
+      <c r="AF52" s="6"/>
       <c r="AG52" s="6"/>
       <c r="AH52" s="6"/>
     </row>
@@ -6982,7 +6975,7 @@
       <c r="F53" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G53" s="21" t="s">
+      <c r="G53" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H53" s="10" t="s">
@@ -7033,16 +7026,16 @@
       <c r="W53" s="10">
         <v>10</v>
       </c>
-      <c r="X53" s="20">
+      <c r="X53" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y53" s="20">
+      <c r="Y53" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z53" s="20">
+      <c r="Z53" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA53" s="20">
+      <c r="AA53" s="18">
         <v>0.1</v>
       </c>
       <c r="AB53" s="10" t="s">
@@ -7051,11 +7044,11 @@
       <c r="AC53" s="10">
         <v>100</v>
       </c>
-      <c r="AD53" s="19" t="s">
+      <c r="AD53" s="17" t="s">
         <v>324</v>
       </c>
-      <c r="AE53" s="14"/>
-      <c r="AF53" s="15"/>
+      <c r="AE53" s="5"/>
+      <c r="AF53" s="6"/>
       <c r="AG53" s="6"/>
       <c r="AH53" s="6"/>
     </row>
@@ -7079,7 +7072,7 @@
       <c r="F54" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="G54" s="21" t="s">
+      <c r="G54" s="19" t="s">
         <v>64</v>
       </c>
       <c r="H54" s="10" t="s">
@@ -7130,16 +7123,16 @@
       <c r="W54" s="10">
         <v>10</v>
       </c>
-      <c r="X54" s="20">
+      <c r="X54" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y54" s="20">
+      <c r="Y54" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z54" s="20">
+      <c r="Z54" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA54" s="20">
+      <c r="AA54" s="18">
         <v>0.1</v>
       </c>
       <c r="AB54" s="10">
@@ -7151,8 +7144,8 @@
       <c r="AD54" s="10" t="s">
         <v>387</v>
       </c>
-      <c r="AE54" s="14"/>
-      <c r="AF54" s="15"/>
+      <c r="AE54" s="5"/>
+      <c r="AF54" s="6"/>
       <c r="AG54" s="6"/>
       <c r="AH54" s="6"/>
     </row>
@@ -7176,7 +7169,7 @@
       <c r="F55" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="G55" s="21" t="s">
+      <c r="G55" s="19" t="s">
         <v>423</v>
       </c>
       <c r="H55" s="10" t="s">
@@ -7197,10 +7190,10 @@
       <c r="M55" s="10">
         <v>200000</v>
       </c>
-      <c r="N55" s="27" t="s">
+      <c r="N55" s="25" t="s">
         <v>301</v>
       </c>
-      <c r="O55" s="27" t="s">
+      <c r="O55" s="25" t="s">
         <v>303</v>
       </c>
       <c r="P55" s="10">
@@ -7227,16 +7220,16 @@
       <c r="W55" s="10">
         <v>10</v>
       </c>
-      <c r="X55" s="20">
+      <c r="X55" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y55" s="20">
+      <c r="Y55" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z55" s="20">
+      <c r="Z55" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA55" s="20">
+      <c r="AA55" s="18">
         <v>0.1</v>
       </c>
       <c r="AB55" s="10">
@@ -7245,11 +7238,11 @@
       <c r="AC55" s="10">
         <v>100</v>
       </c>
-      <c r="AD55" s="22" t="s">
+      <c r="AD55" s="20" t="s">
         <v>424</v>
       </c>
-      <c r="AE55" s="14"/>
-      <c r="AF55" s="15"/>
+      <c r="AE55" s="5"/>
+      <c r="AF55" s="6"/>
       <c r="AG55" s="6"/>
       <c r="AH55" s="6"/>
     </row>
@@ -7272,7 +7265,7 @@
       <c r="F56" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="G56" s="21" t="s">
+      <c r="G56" s="19" t="s">
         <v>64</v>
       </c>
       <c r="H56" s="10" t="s">
@@ -7323,16 +7316,16 @@
       <c r="W56" s="10">
         <v>10</v>
       </c>
-      <c r="X56" s="20">
+      <c r="X56" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y56" s="20">
+      <c r="Y56" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z56" s="20">
+      <c r="Z56" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA56" s="20">
+      <c r="AA56" s="18">
         <v>0.1</v>
       </c>
       <c r="AB56" s="10">
@@ -7344,8 +7337,8 @@
       <c r="AD56" s="10" t="s">
         <v>343</v>
       </c>
-      <c r="AE56" s="14"/>
-      <c r="AF56" s="15"/>
+      <c r="AE56" s="5"/>
+      <c r="AF56" s="6"/>
       <c r="AG56" s="6"/>
       <c r="AH56" s="6"/>
     </row>
@@ -7368,7 +7361,7 @@
       <c r="F57" s="10" t="s">
         <v>342</v>
       </c>
-      <c r="G57" s="21" t="s">
+      <c r="G57" s="19" t="s">
         <v>403</v>
       </c>
       <c r="H57" s="10" t="s">
@@ -7419,16 +7412,16 @@
       <c r="W57" s="10">
         <v>10</v>
       </c>
-      <c r="X57" s="20">
+      <c r="X57" s="18">
         <v>0</v>
       </c>
-      <c r="Y57" s="20">
+      <c r="Y57" s="18">
         <v>0</v>
       </c>
-      <c r="Z57" s="20">
+      <c r="Z57" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA57" s="20">
+      <c r="AA57" s="18">
         <v>0.5</v>
       </c>
       <c r="AB57" s="10">
@@ -7440,8 +7433,8 @@
       <c r="AD57" s="10" t="s">
         <v>409</v>
       </c>
-      <c r="AE57" s="14"/>
-      <c r="AF57" s="15"/>
+      <c r="AE57" s="5"/>
+      <c r="AF57" s="6"/>
       <c r="AG57" s="6"/>
       <c r="AH57" s="6"/>
     </row>
@@ -7464,7 +7457,7 @@
       <c r="F58" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G58" s="21" t="s">
+      <c r="G58" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H58" s="10" t="s">
@@ -7479,7 +7472,7 @@
       <c r="K58" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L58" s="26" t="s">
+      <c r="L58" s="24" t="s">
         <v>61</v>
       </c>
       <c r="M58" s="10" t="s">
@@ -7536,8 +7529,8 @@
       <c r="AD58" s="10" t="s">
         <v>344</v>
       </c>
-      <c r="AE58" s="14"/>
-      <c r="AF58" s="15"/>
+      <c r="AE58" s="5"/>
+      <c r="AF58" s="6"/>
       <c r="AG58" s="6"/>
       <c r="AH58" s="6"/>
     </row>
@@ -7561,7 +7554,7 @@
       <c r="F59" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G59" s="21" t="s">
+      <c r="G59" s="19" t="s">
         <v>313</v>
       </c>
       <c r="H59" s="10" t="s">
@@ -7576,7 +7569,7 @@
       <c r="K59" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L59" s="26" t="s">
+      <c r="L59" s="24" t="s">
         <v>61</v>
       </c>
       <c r="M59" s="10" t="s">
@@ -7594,10 +7587,10 @@
       <c r="Q59" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="R59" s="23" t="s">
+      <c r="R59" s="21" t="s">
         <v>398</v>
       </c>
-      <c r="S59" s="23" t="s">
+      <c r="S59" s="21" t="s">
         <v>398</v>
       </c>
       <c r="T59" s="10">
@@ -7615,13 +7608,13 @@
       <c r="X59" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="Y59" s="20">
+      <c r="Y59" s="18">
         <v>0.1</v>
       </c>
       <c r="Z59" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="AA59" s="20">
+      <c r="AA59" s="18">
         <v>0.1</v>
       </c>
       <c r="AB59" s="10">
@@ -7633,8 +7626,8 @@
       <c r="AD59" s="10" t="s">
         <v>391</v>
       </c>
-      <c r="AE59" s="14"/>
-      <c r="AF59" s="15"/>
+      <c r="AE59" s="5"/>
+      <c r="AF59" s="6"/>
       <c r="AG59" s="6"/>
       <c r="AH59" s="6"/>
     </row>
@@ -7657,7 +7650,7 @@
       <c r="F60" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G60" s="21" t="s">
+      <c r="G60" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H60" s="10" t="s">
@@ -7729,8 +7722,8 @@
       <c r="AD60" s="10" t="s">
         <v>345</v>
       </c>
-      <c r="AE60" s="14"/>
-      <c r="AF60" s="15"/>
+      <c r="AE60" s="5"/>
+      <c r="AF60" s="6"/>
       <c r="AG60" s="6"/>
       <c r="AH60" s="6"/>
     </row>
@@ -7754,7 +7747,7 @@
       <c r="F61" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G61" s="21" t="s">
+      <c r="G61" s="19" t="s">
         <v>64</v>
       </c>
       <c r="H61" s="10" t="s">
@@ -7805,16 +7798,16 @@
       <c r="W61" s="10">
         <v>10</v>
       </c>
-      <c r="X61" s="20">
+      <c r="X61" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y61" s="20">
+      <c r="Y61" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z61" s="20">
+      <c r="Z61" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA61" s="20">
+      <c r="AA61" s="18">
         <v>0.1</v>
       </c>
       <c r="AB61" s="10">
@@ -7826,8 +7819,8 @@
       <c r="AD61" s="10" t="s">
         <v>346</v>
       </c>
-      <c r="AE61" s="14"/>
-      <c r="AF61" s="15"/>
+      <c r="AE61" s="5"/>
+      <c r="AF61" s="6"/>
       <c r="AG61" s="6"/>
       <c r="AH61" s="6"/>
     </row>
@@ -7850,7 +7843,7 @@
       <c r="F62" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G62" s="21" t="s">
+      <c r="G62" s="19" t="s">
         <v>415</v>
       </c>
       <c r="H62" s="10" t="s">
@@ -7901,16 +7894,16 @@
       <c r="W62" s="10">
         <v>10</v>
       </c>
-      <c r="X62" s="20">
+      <c r="X62" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y62" s="20">
+      <c r="Y62" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z62" s="20">
+      <c r="Z62" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA62" s="20">
+      <c r="AA62" s="18">
         <v>0.1</v>
       </c>
       <c r="AB62" s="10" t="s">
@@ -7922,8 +7915,8 @@
       <c r="AD62" s="10" t="s">
         <v>425</v>
       </c>
-      <c r="AE62" s="14"/>
-      <c r="AF62" s="15"/>
+      <c r="AE62" s="5"/>
+      <c r="AF62" s="6"/>
       <c r="AG62" s="6"/>
       <c r="AH62" s="6"/>
     </row>
@@ -7946,7 +7939,7 @@
       <c r="F63" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G63" s="21" t="s">
+      <c r="G63" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H63" s="10" t="s">
@@ -8018,8 +8011,8 @@
       <c r="AD63" s="10" t="s">
         <v>445</v>
       </c>
-      <c r="AE63" s="14"/>
-      <c r="AF63" s="15"/>
+      <c r="AE63" s="5"/>
+      <c r="AF63" s="6"/>
       <c r="AG63" s="6"/>
       <c r="AH63" s="6"/>
     </row>
@@ -8042,7 +8035,7 @@
       <c r="F64" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G64" s="21" t="s">
+      <c r="G64" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H64" s="10" t="s">
@@ -8054,10 +8047,10 @@
       <c r="J64" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K64" s="19" t="s">
+      <c r="K64" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="L64" s="26" t="s">
+      <c r="L64" s="24" t="s">
         <v>61</v>
       </c>
       <c r="M64" s="10" t="s">
@@ -8111,11 +8104,11 @@
       <c r="AC64" s="10">
         <v>100</v>
       </c>
-      <c r="AD64" s="26" t="s">
+      <c r="AD64" s="24" t="s">
         <v>347</v>
       </c>
-      <c r="AE64" s="14"/>
-      <c r="AF64" s="15"/>
+      <c r="AE64" s="5"/>
+      <c r="AF64" s="6"/>
       <c r="AG64" s="6"/>
       <c r="AH64" s="6"/>
     </row>
@@ -8138,7 +8131,7 @@
       <c r="F65" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G65" s="21" t="s">
+      <c r="G65" s="19" t="s">
         <v>64</v>
       </c>
       <c r="H65" s="10" t="s">
@@ -8189,16 +8182,16 @@
       <c r="W65" s="10">
         <v>10</v>
       </c>
-      <c r="X65" s="20">
+      <c r="X65" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y65" s="20">
+      <c r="Y65" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z65" s="20">
+      <c r="Z65" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA65" s="20">
+      <c r="AA65" s="18">
         <v>0.1</v>
       </c>
       <c r="AB65" s="10">
@@ -8210,8 +8203,8 @@
       <c r="AD65" s="10" t="s">
         <v>348</v>
       </c>
-      <c r="AE65" s="14"/>
-      <c r="AF65" s="15"/>
+      <c r="AE65" s="5"/>
+      <c r="AF65" s="6"/>
       <c r="AG65" s="6"/>
       <c r="AH65" s="6"/>
     </row>
@@ -8231,10 +8224,10 @@
       <c r="E66" s="10">
         <v>265</v>
       </c>
-      <c r="F66" s="21" t="s">
+      <c r="F66" s="19" t="s">
         <v>349</v>
       </c>
-      <c r="G66" s="21" t="s">
+      <c r="G66" s="19" t="s">
         <v>64</v>
       </c>
       <c r="H66" s="10" t="s">
@@ -8285,16 +8278,16 @@
       <c r="W66" s="10">
         <v>10</v>
       </c>
-      <c r="X66" s="20">
+      <c r="X66" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y66" s="20">
+      <c r="Y66" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z66" s="20">
+      <c r="Z66" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA66" s="20">
+      <c r="AA66" s="18">
         <v>0.1</v>
       </c>
       <c r="AB66" s="10" t="s">
@@ -8306,8 +8299,8 @@
       <c r="AD66" s="10" t="s">
         <v>426</v>
       </c>
-      <c r="AE66" s="14"/>
-      <c r="AF66" s="15"/>
+      <c r="AE66" s="5"/>
+      <c r="AF66" s="6"/>
       <c r="AG66" s="6"/>
       <c r="AH66" s="6"/>
     </row>
@@ -8327,10 +8320,10 @@
       <c r="E67" s="10">
         <v>265</v>
       </c>
-      <c r="F67" s="26" t="s">
+      <c r="F67" s="24" t="s">
         <v>350</v>
       </c>
-      <c r="G67" s="21" t="s">
+      <c r="G67" s="19" t="s">
         <v>427</v>
       </c>
       <c r="H67" s="10" t="s">
@@ -8342,7 +8335,7 @@
       <c r="J67" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="K67" s="19" t="s">
+      <c r="K67" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L67" s="11" t="s">
@@ -8351,10 +8344,10 @@
       <c r="M67" s="10">
         <v>2000</v>
       </c>
-      <c r="N67" s="27" t="s">
+      <c r="N67" s="25" t="s">
         <v>302</v>
       </c>
-      <c r="O67" s="27" t="s">
+      <c r="O67" s="25" t="s">
         <v>304</v>
       </c>
       <c r="P67" s="10" t="s">
@@ -8363,10 +8356,10 @@
       <c r="Q67" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="R67" s="23" t="s">
+      <c r="R67" s="21" t="s">
         <v>398</v>
       </c>
-      <c r="S67" s="23" t="s">
+      <c r="S67" s="21" t="s">
         <v>398</v>
       </c>
       <c r="T67" s="10">
@@ -8384,13 +8377,13 @@
       <c r="X67" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="Y67" s="20">
+      <c r="Y67" s="18">
         <v>0.1</v>
       </c>
       <c r="Z67" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="AA67" s="20">
+      <c r="AA67" s="18">
         <v>0.1</v>
       </c>
       <c r="AB67" s="10" t="s">
@@ -8402,8 +8395,8 @@
       <c r="AD67" s="13" t="s">
         <v>428</v>
       </c>
-      <c r="AE67" s="14"/>
-      <c r="AF67" s="15"/>
+      <c r="AE67" s="5"/>
+      <c r="AF67" s="6"/>
       <c r="AG67" s="6"/>
       <c r="AH67" s="6"/>
     </row>
@@ -8426,7 +8419,7 @@
       <c r="F68" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G68" s="21" t="s">
+      <c r="G68" s="19" t="s">
         <v>410</v>
       </c>
       <c r="H68" s="10" t="s">
@@ -8498,8 +8491,8 @@
       <c r="AD68" s="10" t="s">
         <v>351</v>
       </c>
-      <c r="AE68" s="14"/>
-      <c r="AF68" s="15"/>
+      <c r="AE68" s="5"/>
+      <c r="AF68" s="6"/>
       <c r="AG68" s="6"/>
       <c r="AH68" s="6"/>
     </row>
@@ -8522,7 +8515,7 @@
       <c r="F69" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G69" s="21" t="s">
+      <c r="G69" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H69" s="10" t="s">
@@ -8594,8 +8587,8 @@
       <c r="AD69" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="AE69" s="14"/>
-      <c r="AF69" s="15"/>
+      <c r="AE69" s="5"/>
+      <c r="AF69" s="6"/>
       <c r="AG69" s="6"/>
       <c r="AH69" s="6"/>
     </row>
@@ -8618,7 +8611,7 @@
       <c r="F70" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G70" s="21" t="s">
+      <c r="G70" s="19" t="s">
         <v>423</v>
       </c>
       <c r="H70" s="10" t="s">
@@ -8630,7 +8623,7 @@
       <c r="J70" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="K70" s="19" t="s">
+      <c r="K70" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L70" s="11" t="s">
@@ -8639,10 +8632,10 @@
       <c r="M70" s="10">
         <v>2000</v>
       </c>
-      <c r="N70" s="27" t="s">
+      <c r="N70" s="25" t="s">
         <v>302</v>
       </c>
-      <c r="O70" s="27" t="s">
+      <c r="O70" s="25" t="s">
         <v>304</v>
       </c>
       <c r="P70" s="10">
@@ -8669,16 +8662,16 @@
       <c r="W70" s="10">
         <v>10</v>
       </c>
-      <c r="X70" s="20">
+      <c r="X70" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y70" s="20">
+      <c r="Y70" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z70" s="20">
+      <c r="Z70" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA70" s="20">
+      <c r="AA70" s="18">
         <v>0.1</v>
       </c>
       <c r="AB70" s="10">
@@ -8690,8 +8683,8 @@
       <c r="AD70" s="10" t="s">
         <v>429</v>
       </c>
-      <c r="AE70" s="14"/>
-      <c r="AF70" s="15"/>
+      <c r="AE70" s="5"/>
+      <c r="AF70" s="6"/>
       <c r="AG70" s="6"/>
       <c r="AH70" s="6"/>
     </row>
@@ -8715,7 +8708,7 @@
       <c r="F71" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G71" s="21" t="s">
+      <c r="G71" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H71" s="10" t="s">
@@ -8787,8 +8780,8 @@
       <c r="AD71" s="10" t="s">
         <v>411</v>
       </c>
-      <c r="AE71" s="14"/>
-      <c r="AF71" s="15"/>
+      <c r="AE71" s="5"/>
+      <c r="AF71" s="6"/>
       <c r="AG71" s="6"/>
       <c r="AH71" s="6"/>
     </row>
@@ -8811,7 +8804,7 @@
       <c r="F72" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G72" s="21" t="s">
+      <c r="G72" s="19" t="s">
         <v>311</v>
       </c>
       <c r="H72" s="10" t="s">
@@ -8823,7 +8816,7 @@
       <c r="J72" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K72" s="19" t="s">
+      <c r="K72" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L72" s="11" t="s">
@@ -8835,7 +8828,7 @@
       <c r="N72" s="10" t="s">
         <v>355</v>
       </c>
-      <c r="O72" s="28" t="s">
+      <c r="O72" s="26" t="s">
         <v>354</v>
       </c>
       <c r="P72" s="10">
@@ -8862,16 +8855,16 @@
       <c r="W72" s="10">
         <v>10</v>
       </c>
-      <c r="X72" s="20">
+      <c r="X72" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y72" s="20">
+      <c r="Y72" s="18">
         <v>0.5</v>
       </c>
-      <c r="Z72" s="20">
+      <c r="Z72" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA72" s="20">
+      <c r="AA72" s="18">
         <v>0.5</v>
       </c>
       <c r="AB72" s="10">
@@ -8883,8 +8876,8 @@
       <c r="AD72" s="13" t="s">
         <v>356</v>
       </c>
-      <c r="AE72" s="14"/>
-      <c r="AF72" s="15"/>
+      <c r="AE72" s="5"/>
+      <c r="AF72" s="6"/>
       <c r="AG72" s="6"/>
       <c r="AH72" s="6"/>
     </row>
@@ -8907,7 +8900,7 @@
       <c r="F73" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G73" s="21" t="s">
+      <c r="G73" s="19" t="s">
         <v>358</v>
       </c>
       <c r="H73" s="10" t="s">
@@ -8979,8 +8972,8 @@
       <c r="AD73" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="AE73" s="14"/>
-      <c r="AF73" s="15"/>
+      <c r="AE73" s="5"/>
+      <c r="AF73" s="6"/>
       <c r="AG73" s="6"/>
       <c r="AH73" s="6"/>
     </row>
@@ -9003,7 +8996,7 @@
       <c r="F74" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G74" s="21" t="s">
+      <c r="G74" s="19" t="s">
         <v>359</v>
       </c>
       <c r="H74" s="10" t="s">
@@ -9054,16 +9047,16 @@
       <c r="W74" s="10">
         <v>10</v>
       </c>
-      <c r="X74" s="20">
+      <c r="X74" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y74" s="20">
+      <c r="Y74" s="18">
         <v>0.2</v>
       </c>
-      <c r="Z74" s="20">
+      <c r="Z74" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA74" s="20">
+      <c r="AA74" s="18">
         <v>0.2</v>
       </c>
       <c r="AB74" s="10" t="s">
@@ -9075,8 +9068,8 @@
       <c r="AD74" s="10" t="s">
         <v>412</v>
       </c>
-      <c r="AE74" s="14"/>
-      <c r="AF74" s="15"/>
+      <c r="AE74" s="5"/>
+      <c r="AF74" s="6"/>
       <c r="AG74" s="6"/>
       <c r="AH74" s="6"/>
     </row>
@@ -9099,7 +9092,7 @@
       <c r="F75" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G75" s="21" t="s">
+      <c r="G75" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H75" s="10" t="s">
@@ -9111,7 +9104,7 @@
       <c r="J75" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K75" s="19" t="s">
+      <c r="K75" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L75" s="11" t="s">
@@ -9150,16 +9143,16 @@
       <c r="W75" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="X75" s="20">
+      <c r="X75" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y75" s="20">
+      <c r="Y75" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z75" s="20">
+      <c r="Z75" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA75" s="20">
+      <c r="AA75" s="18">
         <v>0.1</v>
       </c>
       <c r="AB75" s="10">
@@ -9171,8 +9164,8 @@
       <c r="AD75" s="13" t="s">
         <v>360</v>
       </c>
-      <c r="AE75" s="14"/>
-      <c r="AF75" s="15"/>
+      <c r="AE75" s="5"/>
+      <c r="AF75" s="6"/>
       <c r="AG75" s="6"/>
       <c r="AH75" s="6"/>
     </row>
@@ -9195,7 +9188,7 @@
       <c r="F76" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G76" s="21" t="s">
+      <c r="G76" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H76" s="10" t="s">
@@ -9207,7 +9200,7 @@
       <c r="J76" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K76" s="19" t="s">
+      <c r="K76" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L76" s="11" t="s">
@@ -9267,8 +9260,8 @@
       <c r="AD76" s="10" t="s">
         <v>431</v>
       </c>
-      <c r="AE76" s="14"/>
-      <c r="AF76" s="15"/>
+      <c r="AE76" s="5"/>
+      <c r="AF76" s="6"/>
       <c r="AG76" s="6"/>
       <c r="AH76" s="6"/>
     </row>
@@ -9292,7 +9285,7 @@
       <c r="F77" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G77" s="21" t="s">
+      <c r="G77" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H77" s="10" t="s">
@@ -9364,8 +9357,8 @@
       <c r="AD77" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="AE77" s="14"/>
-      <c r="AF77" s="15"/>
+      <c r="AE77" s="5"/>
+      <c r="AF77" s="6"/>
       <c r="AG77" s="6"/>
       <c r="AH77" s="6"/>
     </row>
@@ -9388,7 +9381,7 @@
       <c r="F78" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G78" s="21" t="s">
+      <c r="G78" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H78" s="10" t="s">
@@ -9460,8 +9453,8 @@
       <c r="AD78" s="10" t="s">
         <v>442</v>
       </c>
-      <c r="AE78" s="14"/>
-      <c r="AF78" s="15"/>
+      <c r="AE78" s="5"/>
+      <c r="AF78" s="6"/>
       <c r="AG78" s="6"/>
       <c r="AH78" s="6"/>
     </row>
@@ -9484,7 +9477,7 @@
       <c r="F79" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G79" s="21" t="s">
+      <c r="G79" s="19" t="s">
         <v>313</v>
       </c>
       <c r="H79" s="10" t="s">
@@ -9517,10 +9510,10 @@
       <c r="Q79" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="R79" s="23" t="s">
+      <c r="R79" s="21" t="s">
         <v>398</v>
       </c>
-      <c r="S79" s="23" t="s">
+      <c r="S79" s="21" t="s">
         <v>398</v>
       </c>
       <c r="T79" s="10">
@@ -9538,13 +9531,13 @@
       <c r="X79" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="Y79" s="20">
+      <c r="Y79" s="18">
         <v>0.1</v>
       </c>
       <c r="Z79" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="AA79" s="20">
+      <c r="AA79" s="18">
         <v>0.1</v>
       </c>
       <c r="AB79" s="10">
@@ -9553,11 +9546,11 @@
       <c r="AC79" s="10">
         <v>100</v>
       </c>
-      <c r="AD79" s="29" t="s">
+      <c r="AD79" s="27" t="s">
         <v>393</v>
       </c>
-      <c r="AE79" s="14"/>
-      <c r="AF79" s="15"/>
+      <c r="AE79" s="5"/>
+      <c r="AF79" s="6"/>
       <c r="AG79" s="6"/>
       <c r="AH79" s="6"/>
     </row>
@@ -9575,12 +9568,12 @@
         <v>60</v>
       </c>
       <c r="E80" s="10">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F80" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G80" s="21" t="s">
+      <c r="G80" s="19" t="s">
         <v>432</v>
       </c>
       <c r="H80" s="10" t="s">
@@ -9631,16 +9624,16 @@
       <c r="W80" s="10">
         <v>10</v>
       </c>
-      <c r="X80" s="20">
+      <c r="X80" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y80" s="20">
+      <c r="Y80" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z80" s="20">
+      <c r="Z80" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA80" s="20">
+      <c r="AA80" s="18">
         <v>0.1</v>
       </c>
       <c r="AB80" s="10">
@@ -9652,8 +9645,8 @@
       <c r="AD80" s="10" t="s">
         <v>433</v>
       </c>
-      <c r="AE80" s="14"/>
-      <c r="AF80" s="15"/>
+      <c r="AE80" s="5"/>
+      <c r="AF80" s="6"/>
       <c r="AG80" s="6"/>
       <c r="AH80" s="6"/>
     </row>
@@ -9676,7 +9669,7 @@
       <c r="F81" s="13" t="s">
         <v>366</v>
       </c>
-      <c r="G81" s="21" t="s">
+      <c r="G81" s="19" t="s">
         <v>311</v>
       </c>
       <c r="H81" s="10" t="s">
@@ -9688,7 +9681,7 @@
       <c r="J81" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K81" s="19" t="s">
+      <c r="K81" s="17" t="s">
         <v>319</v>
       </c>
       <c r="L81" s="13" t="s">
@@ -9709,10 +9702,10 @@
       <c r="Q81" s="10" t="s">
         <v>364</v>
       </c>
-      <c r="R81" s="23" t="s">
+      <c r="R81" s="21" t="s">
         <v>365</v>
       </c>
-      <c r="S81" s="23" t="s">
+      <c r="S81" s="21" t="s">
         <v>365</v>
       </c>
       <c r="T81" s="10">
@@ -9727,19 +9720,19 @@
       <c r="W81" s="10">
         <v>10</v>
       </c>
-      <c r="X81" s="20">
+      <c r="X81" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y81" s="20">
+      <c r="Y81" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z81" s="20">
+      <c r="Z81" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA81" s="20">
+      <c r="AA81" s="18">
         <v>0.1</v>
       </c>
-      <c r="AB81" s="30">
+      <c r="AB81" s="28">
         <v>6</v>
       </c>
       <c r="AC81" s="10">
@@ -9748,8 +9741,8 @@
       <c r="AD81" s="13" t="s">
         <v>369</v>
       </c>
-      <c r="AE81" s="14"/>
-      <c r="AF81" s="15"/>
+      <c r="AE81" s="5"/>
+      <c r="AF81" s="6"/>
       <c r="AG81" s="6"/>
       <c r="AH81" s="6"/>
     </row>
@@ -9772,7 +9765,7 @@
       <c r="F82" s="13" t="s">
         <v>367</v>
       </c>
-      <c r="G82" s="21" t="s">
+      <c r="G82" s="19" t="s">
         <v>311</v>
       </c>
       <c r="H82" s="10" t="s">
@@ -9784,7 +9777,7 @@
       <c r="J82" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K82" s="19" t="s">
+      <c r="K82" s="17" t="s">
         <v>319</v>
       </c>
       <c r="L82" s="13" t="s">
@@ -9805,10 +9798,10 @@
       <c r="Q82" s="10">
         <v>100</v>
       </c>
-      <c r="R82" s="23">
+      <c r="R82" s="21">
         <v>0</v>
       </c>
-      <c r="S82" s="23">
+      <c r="S82" s="21">
         <v>0</v>
       </c>
       <c r="T82" s="10">
@@ -9823,19 +9816,19 @@
       <c r="W82" s="10">
         <v>10</v>
       </c>
-      <c r="X82" s="20">
+      <c r="X82" s="18">
         <v>1</v>
       </c>
-      <c r="Y82" s="20">
+      <c r="Y82" s="18">
         <v>1</v>
       </c>
-      <c r="Z82" s="20">
+      <c r="Z82" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA82" s="20">
+      <c r="AA82" s="18">
         <v>0.5</v>
       </c>
-      <c r="AB82" s="30">
+      <c r="AB82" s="28">
         <v>6</v>
       </c>
       <c r="AC82" s="10">
@@ -9844,8 +9837,8 @@
       <c r="AD82" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="AE82" s="14"/>
-      <c r="AF82" s="15"/>
+      <c r="AE82" s="5"/>
+      <c r="AF82" s="6"/>
       <c r="AG82" s="6"/>
       <c r="AH82" s="6"/>
     </row>
@@ -9868,7 +9861,7 @@
       <c r="F83" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G83" s="21" t="s">
+      <c r="G83" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H83" s="10" t="s">
@@ -9940,8 +9933,8 @@
       <c r="AD83" s="10" t="s">
         <v>371</v>
       </c>
-      <c r="AE83" s="14"/>
-      <c r="AF83" s="15"/>
+      <c r="AE83" s="5"/>
+      <c r="AF83" s="6"/>
       <c r="AG83" s="6"/>
       <c r="AH83" s="6"/>
     </row>
@@ -9964,7 +9957,7 @@
       <c r="F84" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G84" s="21" t="s">
+      <c r="G84" s="19" t="s">
         <v>372</v>
       </c>
       <c r="H84" s="10" t="s">
@@ -10036,8 +10029,8 @@
       <c r="AD84" s="10" t="s">
         <v>413</v>
       </c>
-      <c r="AE84" s="14"/>
-      <c r="AF84" s="15"/>
+      <c r="AE84" s="5"/>
+      <c r="AF84" s="6"/>
       <c r="AG84" s="6"/>
       <c r="AH84" s="6"/>
     </row>
@@ -10060,7 +10053,7 @@
       <c r="F85" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G85" s="21" t="s">
+      <c r="G85" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H85" s="10" t="s">
@@ -10132,8 +10125,8 @@
       <c r="AD85" s="10" t="s">
         <v>373</v>
       </c>
-      <c r="AE85" s="14"/>
-      <c r="AF85" s="15"/>
+      <c r="AE85" s="5"/>
+      <c r="AF85" s="6"/>
       <c r="AG85" s="6"/>
       <c r="AH85" s="6"/>
     </row>
@@ -10156,7 +10149,7 @@
       <c r="F86" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G86" s="21" t="s">
+      <c r="G86" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H86" s="10" t="s">
@@ -10228,8 +10221,8 @@
       <c r="AD86" s="10" t="s">
         <v>388</v>
       </c>
-      <c r="AE86" s="14"/>
-      <c r="AF86" s="15"/>
+      <c r="AE86" s="5"/>
+      <c r="AF86" s="6"/>
       <c r="AG86" s="6"/>
       <c r="AH86" s="6"/>
     </row>
@@ -10252,7 +10245,7 @@
       <c r="F87" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G87" s="21" t="s">
+      <c r="G87" s="19" t="s">
         <v>311</v>
       </c>
       <c r="H87" s="10" t="s">
@@ -10303,29 +10296,29 @@
       <c r="W87" s="10">
         <v>10</v>
       </c>
-      <c r="X87" s="20">
+      <c r="X87" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y87" s="20">
+      <c r="Y87" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z87" s="20">
+      <c r="Z87" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA87" s="20">
+      <c r="AA87" s="18">
         <v>0.1</v>
       </c>
       <c r="AB87" s="10">
         <v>10</v>
       </c>
-      <c r="AC87" s="30">
+      <c r="AC87" s="28">
         <v>400</v>
       </c>
       <c r="AD87" s="13" t="s">
         <v>305</v>
       </c>
-      <c r="AE87" s="14"/>
-      <c r="AF87" s="15"/>
+      <c r="AE87" s="5"/>
+      <c r="AF87" s="6"/>
       <c r="AG87" s="6"/>
       <c r="AH87" s="6"/>
     </row>
@@ -10349,7 +10342,7 @@
       <c r="F88" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G88" s="21" t="s">
+      <c r="G88" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H88" s="10" t="s">
@@ -10421,8 +10414,8 @@
       <c r="AD88" s="10" t="s">
         <v>374</v>
       </c>
-      <c r="AE88" s="14"/>
-      <c r="AF88" s="15"/>
+      <c r="AE88" s="5"/>
+      <c r="AF88" s="6"/>
       <c r="AG88" s="6"/>
       <c r="AH88" s="6"/>
     </row>
@@ -10446,7 +10439,7 @@
       <c r="F89" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G89" s="21" t="s">
+      <c r="G89" s="19" t="s">
         <v>311</v>
       </c>
       <c r="H89" s="10" t="s">
@@ -10497,16 +10490,16 @@
       <c r="W89" s="10">
         <v>10</v>
       </c>
-      <c r="X89" s="20">
+      <c r="X89" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y89" s="20">
+      <c r="Y89" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z89" s="20">
+      <c r="Z89" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA89" s="20">
+      <c r="AA89" s="18">
         <v>0.1</v>
       </c>
       <c r="AB89" s="10">
@@ -10518,8 +10511,8 @@
       <c r="AD89" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="AE89" s="14"/>
-      <c r="AF89" s="15"/>
+      <c r="AE89" s="5"/>
+      <c r="AF89" s="6"/>
       <c r="AG89" s="6"/>
       <c r="AH89" s="6"/>
     </row>
@@ -10543,7 +10536,7 @@
       <c r="F90" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G90" s="21" t="s">
+      <c r="G90" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H90" s="10" t="s">
@@ -10615,8 +10608,8 @@
       <c r="AD90" s="10" t="s">
         <v>434</v>
       </c>
-      <c r="AE90" s="14"/>
-      <c r="AF90" s="15"/>
+      <c r="AE90" s="5"/>
+      <c r="AF90" s="6"/>
       <c r="AG90" s="6"/>
       <c r="AH90" s="6"/>
     </row>
@@ -10640,7 +10633,7 @@
       <c r="F91" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G91" s="21" t="s">
+      <c r="G91" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H91" s="10" t="s">
@@ -10712,8 +10705,8 @@
       <c r="AD91" s="10" t="s">
         <v>375</v>
       </c>
-      <c r="AE91" s="14"/>
-      <c r="AF91" s="15"/>
+      <c r="AE91" s="5"/>
+      <c r="AF91" s="6"/>
       <c r="AG91" s="6"/>
       <c r="AH91" s="6"/>
     </row>
@@ -10737,7 +10730,7 @@
       <c r="F92" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G92" s="21" t="s">
+      <c r="G92" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H92" s="10" t="s">
@@ -10809,8 +10802,8 @@
       <c r="AD92" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="AE92" s="14"/>
-      <c r="AF92" s="15"/>
+      <c r="AE92" s="5"/>
+      <c r="AF92" s="6"/>
       <c r="AG92" s="6"/>
       <c r="AH92" s="6"/>
     </row>
@@ -10833,7 +10826,7 @@
       <c r="F93" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G93" s="21" t="s">
+      <c r="G93" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H93" s="10" t="s">
@@ -10845,10 +10838,10 @@
       <c r="J93" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K93" s="19" t="s">
+      <c r="K93" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="L93" s="29" t="s">
+      <c r="L93" s="27" t="s">
         <v>61</v>
       </c>
       <c r="M93" s="10" t="s">
@@ -10905,8 +10898,8 @@
       <c r="AD93" s="10" t="s">
         <v>377</v>
       </c>
-      <c r="AE93" s="14"/>
-      <c r="AF93" s="15"/>
+      <c r="AE93" s="5"/>
+      <c r="AF93" s="6"/>
       <c r="AG93" s="6"/>
       <c r="AH93" s="6"/>
     </row>
@@ -10930,7 +10923,7 @@
       <c r="F94" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G94" s="21" t="s">
+      <c r="G94" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H94" s="10" t="s">
@@ -11002,8 +10995,8 @@
       <c r="AD94" s="10" t="s">
         <v>378</v>
       </c>
-      <c r="AE94" s="14"/>
-      <c r="AF94" s="15"/>
+      <c r="AE94" s="5"/>
+      <c r="AF94" s="6"/>
       <c r="AG94" s="6"/>
       <c r="AH94" s="6"/>
     </row>
@@ -11027,7 +11020,7 @@
       <c r="F95" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G95" s="21" t="s">
+      <c r="G95" s="19" t="s">
         <v>437</v>
       </c>
       <c r="H95" s="10" t="s">
@@ -11042,7 +11035,7 @@
       <c r="K95" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L95" s="29" t="s">
+      <c r="L95" s="27" t="s">
         <v>306</v>
       </c>
       <c r="M95" s="10">
@@ -11078,16 +11071,16 @@
       <c r="W95" s="10">
         <v>10</v>
       </c>
-      <c r="X95" s="20">
+      <c r="X95" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y95" s="20">
+      <c r="Y95" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z95" s="20">
+      <c r="Z95" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA95" s="20">
+      <c r="AA95" s="18">
         <v>0.1</v>
       </c>
       <c r="AB95" s="10">
@@ -11099,8 +11092,8 @@
       <c r="AD95" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="AE95" s="14"/>
-      <c r="AF95" s="15"/>
+      <c r="AE95" s="5"/>
+      <c r="AF95" s="6"/>
       <c r="AG95" s="6"/>
       <c r="AH95" s="6"/>
     </row>
@@ -11123,7 +11116,7 @@
       <c r="F96" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G96" s="21" t="s">
+      <c r="G96" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H96" s="10" t="s">
@@ -11135,7 +11128,7 @@
       <c r="J96" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K96" s="19" t="s">
+      <c r="K96" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L96" s="11" t="s">
@@ -11174,16 +11167,16 @@
       <c r="W96" s="10">
         <v>10</v>
       </c>
-      <c r="X96" s="20">
+      <c r="X96" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y96" s="20">
+      <c r="Y96" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z96" s="20">
+      <c r="Z96" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA96" s="20">
+      <c r="AA96" s="18">
         <v>0.1</v>
       </c>
       <c r="AB96" s="10">
@@ -11195,8 +11188,8 @@
       <c r="AD96" s="10" t="s">
         <v>390</v>
       </c>
-      <c r="AE96" s="14"/>
-      <c r="AF96" s="15"/>
+      <c r="AE96" s="5"/>
+      <c r="AF96" s="6"/>
       <c r="AG96" s="6"/>
       <c r="AH96" s="6"/>
     </row>
@@ -11219,7 +11212,7 @@
       <c r="F97" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G97" s="21" t="s">
+      <c r="G97" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H97" s="10" t="s">
@@ -11231,7 +11224,7 @@
       <c r="J97" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K97" s="19" t="s">
+      <c r="K97" s="17" t="s">
         <v>319</v>
       </c>
       <c r="L97" s="10" t="s">
@@ -11270,16 +11263,16 @@
       <c r="W97" s="10">
         <v>10</v>
       </c>
-      <c r="X97" s="20">
+      <c r="X97" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y97" s="20">
+      <c r="Y97" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z97" s="20">
+      <c r="Z97" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA97" s="20">
+      <c r="AA97" s="18">
         <v>0.1</v>
       </c>
       <c r="AB97" s="10">
@@ -11288,11 +11281,11 @@
       <c r="AC97" s="10">
         <v>100</v>
       </c>
-      <c r="AD97" s="31" t="s">
+      <c r="AD97" s="29" t="s">
         <v>443</v>
       </c>
-      <c r="AE97" s="14"/>
-      <c r="AF97" s="15"/>
+      <c r="AE97" s="5"/>
+      <c r="AF97" s="6"/>
       <c r="AG97" s="6"/>
       <c r="AH97" s="6"/>
     </row>
@@ -11315,7 +11308,7 @@
       <c r="F98" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G98" s="21" t="s">
+      <c r="G98" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H98" s="10" t="s">
@@ -11330,7 +11323,7 @@
       <c r="K98" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="L98" s="29" t="s">
+      <c r="L98" s="27" t="s">
         <v>61</v>
       </c>
       <c r="M98" s="10" t="s">
@@ -11387,8 +11380,8 @@
       <c r="AD98" s="10" t="s">
         <v>379</v>
       </c>
-      <c r="AE98" s="14"/>
-      <c r="AF98" s="15"/>
+      <c r="AE98" s="5"/>
+      <c r="AF98" s="6"/>
       <c r="AG98" s="6"/>
       <c r="AH98" s="6"/>
     </row>
@@ -11412,7 +11405,7 @@
       <c r="F99" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G99" s="21" t="s">
+      <c r="G99" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H99" s="10" t="s">
@@ -11484,8 +11477,8 @@
       <c r="AD99" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="AE99" s="14"/>
-      <c r="AF99" s="15"/>
+      <c r="AE99" s="5"/>
+      <c r="AF99" s="6"/>
       <c r="AG99" s="6"/>
       <c r="AH99" s="6"/>
     </row>
@@ -11508,7 +11501,7 @@
       <c r="F100" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G100" s="21" t="s">
+      <c r="G100" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H100" s="10" t="s">
@@ -11520,10 +11513,10 @@
       <c r="J100" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K100" s="19" t="s">
+      <c r="K100" s="17" t="s">
         <v>315</v>
       </c>
-      <c r="L100" s="29" t="s">
+      <c r="L100" s="27" t="s">
         <v>61</v>
       </c>
       <c r="M100" s="10" t="s">
@@ -11580,8 +11573,8 @@
       <c r="AD100" s="10" t="s">
         <v>381</v>
       </c>
-      <c r="AE100" s="14"/>
-      <c r="AF100" s="15"/>
+      <c r="AE100" s="5"/>
+      <c r="AF100" s="6"/>
       <c r="AG100" s="6"/>
       <c r="AH100" s="6"/>
     </row>
@@ -11604,7 +11597,7 @@
       <c r="F101" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G101" s="21" t="s">
+      <c r="G101" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H101" s="10" t="s">
@@ -11616,10 +11609,10 @@
       <c r="J101" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K101" s="19" t="s">
+      <c r="K101" s="17" t="s">
         <v>315</v>
       </c>
-      <c r="L101" s="29" t="s">
+      <c r="L101" s="27" t="s">
         <v>61</v>
       </c>
       <c r="M101" s="10" t="s">
@@ -11676,8 +11669,8 @@
       <c r="AD101" s="10" t="s">
         <v>446</v>
       </c>
-      <c r="AE101" s="14"/>
-      <c r="AF101" s="15"/>
+      <c r="AE101" s="5"/>
+      <c r="AF101" s="6"/>
       <c r="AG101" s="6"/>
       <c r="AH101" s="6"/>
     </row>
@@ -11700,7 +11693,7 @@
       <c r="F102" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G102" s="21" t="s">
+      <c r="G102" s="19" t="s">
         <v>313</v>
       </c>
       <c r="H102" s="10" t="s">
@@ -11712,7 +11705,7 @@
       <c r="J102" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K102" s="19" t="s">
+      <c r="K102" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L102" s="10" t="s">
@@ -11733,10 +11726,10 @@
       <c r="Q102" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="R102" s="23" t="s">
+      <c r="R102" s="21" t="s">
         <v>398</v>
       </c>
-      <c r="S102" s="23" t="s">
+      <c r="S102" s="21" t="s">
         <v>398</v>
       </c>
       <c r="T102" s="10">
@@ -11754,13 +11747,13 @@
       <c r="X102" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="Y102" s="20">
+      <c r="Y102" s="18">
         <v>0.1</v>
       </c>
       <c r="Z102" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="AA102" s="20">
+      <c r="AA102" s="18">
         <v>0.1</v>
       </c>
       <c r="AB102" s="10" t="s">
@@ -11772,8 +11765,8 @@
       <c r="AD102" s="10" t="s">
         <v>394</v>
       </c>
-      <c r="AE102" s="14"/>
-      <c r="AF102" s="15"/>
+      <c r="AE102" s="5"/>
+      <c r="AF102" s="6"/>
       <c r="AG102" s="6"/>
       <c r="AH102" s="6"/>
     </row>
@@ -11796,7 +11789,7 @@
       <c r="F103" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G103" s="21" t="s">
+      <c r="G103" s="19" t="s">
         <v>414</v>
       </c>
       <c r="H103" s="10" t="s">
@@ -11808,10 +11801,10 @@
       <c r="J103" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K103" s="19" t="s">
+      <c r="K103" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="L103" s="29" t="s">
+      <c r="L103" s="27" t="s">
         <v>297</v>
       </c>
       <c r="M103" s="10">
@@ -11847,16 +11840,16 @@
       <c r="W103" s="10">
         <v>10</v>
       </c>
-      <c r="X103" s="20">
+      <c r="X103" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y103" s="20">
+      <c r="Y103" s="18">
         <v>0.5</v>
       </c>
-      <c r="Z103" s="20">
+      <c r="Z103" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA103" s="20">
+      <c r="AA103" s="18">
         <v>0.5</v>
       </c>
       <c r="AB103" s="10">
@@ -11865,11 +11858,11 @@
       <c r="AC103" s="10">
         <v>80</v>
       </c>
-      <c r="AD103" s="31" t="s">
+      <c r="AD103" s="29" t="s">
         <v>444</v>
       </c>
-      <c r="AE103" s="14"/>
-      <c r="AF103" s="15"/>
+      <c r="AE103" s="5"/>
+      <c r="AF103" s="6"/>
       <c r="AG103" s="6"/>
       <c r="AH103" s="6"/>
     </row>
@@ -11892,7 +11885,7 @@
       <c r="F104" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G104" s="21" t="s">
+      <c r="G104" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H104" s="10" t="s">
@@ -11904,7 +11897,7 @@
       <c r="J104" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="K104" s="19" t="s">
+      <c r="K104" s="17" t="s">
         <v>319</v>
       </c>
       <c r="L104" s="11" t="s">
@@ -11964,8 +11957,8 @@
       <c r="AD104" s="10" t="s">
         <v>435</v>
       </c>
-      <c r="AE104" s="14"/>
-      <c r="AF104" s="15"/>
+      <c r="AE104" s="5"/>
+      <c r="AF104" s="6"/>
       <c r="AG104" s="6"/>
       <c r="AH104" s="6"/>
     </row>
@@ -11989,7 +11982,7 @@
       <c r="F105" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G105" s="21" t="s">
+      <c r="G105" s="19" t="s">
         <v>432</v>
       </c>
       <c r="H105" s="10" t="s">
@@ -12001,7 +11994,7 @@
       <c r="J105" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="K105" s="19" t="s">
+      <c r="K105" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L105" s="11" t="s">
@@ -12040,16 +12033,16 @@
       <c r="W105" s="10">
         <v>10</v>
       </c>
-      <c r="X105" s="20">
+      <c r="X105" s="18">
         <v>0.5</v>
       </c>
-      <c r="Y105" s="20">
+      <c r="Y105" s="18">
         <v>0.1</v>
       </c>
-      <c r="Z105" s="20">
+      <c r="Z105" s="18">
         <v>0.5</v>
       </c>
-      <c r="AA105" s="20">
+      <c r="AA105" s="18">
         <v>0.1</v>
       </c>
       <c r="AB105" s="10">
@@ -12061,8 +12054,8 @@
       <c r="AD105" s="10" t="s">
         <v>436</v>
       </c>
-      <c r="AE105" s="14"/>
-      <c r="AF105" s="15"/>
+      <c r="AE105" s="5"/>
+      <c r="AF105" s="6"/>
       <c r="AG105" s="6"/>
       <c r="AH105" s="6"/>
     </row>
@@ -12085,7 +12078,7 @@
       <c r="F106" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G106" s="21" t="s">
+      <c r="G106" s="19" t="s">
         <v>61</v>
       </c>
       <c r="H106" s="10" t="s">
@@ -12097,7 +12090,7 @@
       <c r="J106" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K106" s="19" t="s">
+      <c r="K106" s="17" t="s">
         <v>315</v>
       </c>
       <c r="L106" s="11" t="s">
@@ -12157,584 +12150,311 @@
       <c r="AD106" s="10" t="s">
         <v>382</v>
       </c>
-      <c r="AE106" s="14"/>
-      <c r="AF106" s="15"/>
+      <c r="AE106" s="5"/>
+      <c r="AF106" s="6"/>
       <c r="AG106" s="6"/>
       <c r="AH106" s="6"/>
     </row>
     <row r="107" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="32"/>
-      <c r="B107" s="32"/>
-      <c r="C107" s="32"/>
-      <c r="D107" s="14"/>
-      <c r="E107" s="14"/>
-      <c r="F107" s="14"/>
-      <c r="G107" s="14"/>
-      <c r="H107" s="14"/>
-      <c r="I107" s="14"/>
-      <c r="J107" s="14"/>
-      <c r="K107" s="14"/>
-      <c r="L107" s="32"/>
-      <c r="M107" s="14"/>
-      <c r="N107" s="32"/>
-      <c r="O107" s="32"/>
-      <c r="P107" s="32"/>
-      <c r="Q107" s="32"/>
-      <c r="R107" s="32"/>
-      <c r="S107" s="32"/>
-      <c r="T107" s="32"/>
-      <c r="U107" s="32"/>
-      <c r="V107" s="32"/>
-      <c r="W107" s="32"/>
-      <c r="X107" s="32"/>
-      <c r="Y107" s="32"/>
-      <c r="Z107" s="32"/>
-      <c r="AA107" s="32"/>
-      <c r="AB107" s="32"/>
-      <c r="AC107" s="14"/>
-      <c r="AD107" s="14"/>
-      <c r="AE107" s="14"/>
-      <c r="AF107" s="15"/>
+      <c r="D107" s="5"/>
+      <c r="E107" s="5"/>
+      <c r="F107" s="5"/>
+      <c r="G107" s="5"/>
+      <c r="H107" s="5"/>
+      <c r="I107" s="5"/>
+      <c r="J107" s="5"/>
+      <c r="K107" s="5"/>
+      <c r="M107" s="5"/>
+      <c r="AC107" s="5"/>
+      <c r="AD107" s="5"/>
+      <c r="AE107" s="5"/>
+      <c r="AF107" s="6"/>
       <c r="AG107" s="6"/>
       <c r="AH107" s="6"/>
     </row>
     <row r="108" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="32"/>
-      <c r="B108" s="32"/>
-      <c r="C108" s="32"/>
-      <c r="D108" s="14"/>
-      <c r="E108" s="14"/>
-      <c r="F108" s="14"/>
-      <c r="G108" s="14"/>
-      <c r="H108" s="14"/>
-      <c r="I108" s="14"/>
-      <c r="J108" s="14"/>
-      <c r="K108" s="14"/>
-      <c r="L108" s="32"/>
-      <c r="M108" s="14"/>
-      <c r="N108" s="32"/>
-      <c r="O108" s="32"/>
-      <c r="P108" s="32"/>
-      <c r="Q108" s="32"/>
-      <c r="R108" s="32"/>
-      <c r="S108" s="32"/>
-      <c r="T108" s="32"/>
-      <c r="U108" s="32"/>
-      <c r="V108" s="32"/>
-      <c r="W108" s="32"/>
-      <c r="X108" s="32"/>
-      <c r="Y108" s="32"/>
-      <c r="Z108" s="32"/>
-      <c r="AA108" s="32"/>
-      <c r="AB108" s="32"/>
-      <c r="AC108" s="14"/>
-      <c r="AD108" s="14"/>
-      <c r="AE108" s="14"/>
-      <c r="AF108" s="15"/>
+      <c r="D108" s="5"/>
+      <c r="E108" s="5"/>
+      <c r="F108" s="5"/>
+      <c r="G108" s="5"/>
+      <c r="H108" s="5"/>
+      <c r="I108" s="5"/>
+      <c r="J108" s="5"/>
+      <c r="K108" s="5"/>
+      <c r="M108" s="5"/>
+      <c r="AC108" s="5"/>
+      <c r="AD108" s="5"/>
+      <c r="AE108" s="5"/>
+      <c r="AF108" s="6"/>
       <c r="AG108" s="6"/>
       <c r="AH108" s="6"/>
     </row>
     <row r="109" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="32"/>
-      <c r="B109" s="32"/>
-      <c r="C109" s="32"/>
-      <c r="D109" s="14"/>
-      <c r="E109" s="14"/>
-      <c r="F109" s="14"/>
-      <c r="G109" s="14"/>
-      <c r="H109" s="14"/>
-      <c r="I109" s="14"/>
-      <c r="J109" s="14"/>
-      <c r="K109" s="14"/>
-      <c r="L109" s="32"/>
-      <c r="M109" s="14"/>
-      <c r="N109" s="32"/>
-      <c r="O109" s="32"/>
-      <c r="P109" s="32"/>
-      <c r="Q109" s="32"/>
-      <c r="R109" s="32"/>
-      <c r="S109" s="32"/>
-      <c r="T109" s="32"/>
-      <c r="U109" s="32"/>
-      <c r="V109" s="32"/>
-      <c r="W109" s="32"/>
-      <c r="X109" s="32"/>
-      <c r="Y109" s="32"/>
-      <c r="Z109" s="32"/>
-      <c r="AA109" s="32"/>
-      <c r="AB109" s="32"/>
-      <c r="AC109" s="14"/>
-      <c r="AD109" s="14"/>
-      <c r="AE109" s="14"/>
-      <c r="AF109" s="15"/>
+      <c r="D109" s="5"/>
+      <c r="E109" s="5"/>
+      <c r="F109" s="5"/>
+      <c r="G109" s="5"/>
+      <c r="H109" s="5"/>
+      <c r="I109" s="5"/>
+      <c r="J109" s="5"/>
+      <c r="K109" s="5"/>
+      <c r="M109" s="5"/>
+      <c r="AC109" s="5"/>
+      <c r="AD109" s="5"/>
+      <c r="AE109" s="5"/>
+      <c r="AF109" s="6"/>
       <c r="AG109" s="6"/>
       <c r="AH109" s="6"/>
     </row>
     <row r="110" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="32"/>
-      <c r="B110" s="32"/>
-      <c r="C110" s="32"/>
-      <c r="D110" s="14"/>
-      <c r="E110" s="14"/>
-      <c r="F110" s="14"/>
-      <c r="G110" s="14"/>
-      <c r="H110" s="14"/>
-      <c r="I110" s="14"/>
-      <c r="J110" s="14"/>
-      <c r="K110" s="14"/>
-      <c r="L110" s="32"/>
-      <c r="M110" s="14"/>
-      <c r="N110" s="32"/>
-      <c r="O110" s="32"/>
-      <c r="P110" s="32"/>
-      <c r="Q110" s="32"/>
-      <c r="R110" s="32"/>
-      <c r="S110" s="32"/>
-      <c r="T110" s="32"/>
-      <c r="U110" s="32"/>
-      <c r="V110" s="32"/>
-      <c r="W110" s="32"/>
-      <c r="X110" s="32"/>
-      <c r="Y110" s="32"/>
-      <c r="Z110" s="32"/>
-      <c r="AA110" s="32"/>
-      <c r="AB110" s="32"/>
-      <c r="AC110" s="14"/>
-      <c r="AD110" s="14"/>
-      <c r="AE110" s="14"/>
-      <c r="AF110" s="15"/>
+      <c r="D110" s="5"/>
+      <c r="E110" s="5"/>
+      <c r="F110" s="5"/>
+      <c r="G110" s="5"/>
+      <c r="H110" s="5"/>
+      <c r="I110" s="5"/>
+      <c r="J110" s="5"/>
+      <c r="K110" s="5"/>
+      <c r="M110" s="5"/>
+      <c r="AC110" s="5"/>
+      <c r="AD110" s="5"/>
+      <c r="AE110" s="5"/>
+      <c r="AF110" s="6"/>
       <c r="AG110" s="6"/>
       <c r="AH110" s="6"/>
     </row>
     <row r="111" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="32"/>
-      <c r="B111" s="32"/>
-      <c r="C111" s="32"/>
-      <c r="D111" s="14"/>
-      <c r="E111" s="14"/>
-      <c r="F111" s="14"/>
-      <c r="G111" s="14"/>
-      <c r="H111" s="14"/>
-      <c r="I111" s="14"/>
-      <c r="J111" s="14"/>
-      <c r="K111" s="14"/>
-      <c r="L111" s="32"/>
-      <c r="M111" s="14"/>
-      <c r="N111" s="32"/>
-      <c r="O111" s="32"/>
-      <c r="P111" s="32"/>
-      <c r="Q111" s="32"/>
-      <c r="R111" s="32"/>
-      <c r="S111" s="32"/>
-      <c r="T111" s="32"/>
-      <c r="U111" s="32"/>
-      <c r="V111" s="32"/>
-      <c r="W111" s="32"/>
-      <c r="X111" s="32"/>
-      <c r="Y111" s="32"/>
-      <c r="Z111" s="32"/>
-      <c r="AA111" s="32"/>
-      <c r="AB111" s="14"/>
-      <c r="AC111" s="14"/>
-      <c r="AD111" s="14"/>
-      <c r="AE111" s="14"/>
-      <c r="AF111" s="15"/>
+      <c r="D111" s="5"/>
+      <c r="E111" s="5"/>
+      <c r="F111" s="5"/>
+      <c r="G111" s="5"/>
+      <c r="H111" s="5"/>
+      <c r="I111" s="5"/>
+      <c r="J111" s="5"/>
+      <c r="K111" s="5"/>
+      <c r="M111" s="5"/>
+      <c r="AB111" s="5"/>
+      <c r="AC111" s="5"/>
+      <c r="AD111" s="5"/>
+      <c r="AE111" s="5"/>
+      <c r="AF111" s="6"/>
       <c r="AG111" s="6"/>
       <c r="AH111" s="6"/>
     </row>
     <row r="112" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="32"/>
-      <c r="B112" s="32"/>
-      <c r="C112" s="32"/>
-      <c r="D112" s="14"/>
-      <c r="E112" s="14"/>
-      <c r="F112" s="14"/>
-      <c r="G112" s="14"/>
-      <c r="H112" s="14"/>
-      <c r="I112" s="14"/>
-      <c r="J112" s="14"/>
-      <c r="K112" s="14"/>
-      <c r="L112" s="32"/>
-      <c r="M112" s="14"/>
-      <c r="N112" s="32"/>
-      <c r="O112" s="32"/>
-      <c r="P112" s="32"/>
-      <c r="Q112" s="32"/>
-      <c r="R112" s="32"/>
-      <c r="S112" s="32"/>
-      <c r="T112" s="32"/>
-      <c r="U112" s="32"/>
-      <c r="V112" s="32"/>
-      <c r="W112" s="32"/>
-      <c r="X112" s="32"/>
-      <c r="Y112" s="32"/>
-      <c r="Z112" s="32"/>
-      <c r="AA112" s="32"/>
-      <c r="AB112" s="14"/>
-      <c r="AC112" s="14"/>
-      <c r="AD112" s="14"/>
-      <c r="AE112" s="14"/>
-      <c r="AF112" s="15"/>
+      <c r="D112" s="5"/>
+      <c r="E112" s="5"/>
+      <c r="F112" s="5"/>
+      <c r="G112" s="5"/>
+      <c r="H112" s="5"/>
+      <c r="I112" s="5"/>
+      <c r="J112" s="5"/>
+      <c r="K112" s="5"/>
+      <c r="M112" s="5"/>
+      <c r="AB112" s="5"/>
+      <c r="AC112" s="5"/>
+      <c r="AD112" s="5"/>
+      <c r="AE112" s="5"/>
+      <c r="AF112" s="6"/>
       <c r="AG112" s="6"/>
       <c r="AH112" s="6"/>
     </row>
     <row r="113" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="32"/>
-      <c r="B113" s="32"/>
-      <c r="C113" s="32"/>
-      <c r="D113" s="14"/>
-      <c r="E113" s="14"/>
-      <c r="F113" s="14"/>
-      <c r="G113" s="14"/>
-      <c r="H113" s="14"/>
-      <c r="I113" s="14"/>
-      <c r="J113" s="14"/>
-      <c r="K113" s="14"/>
-      <c r="L113" s="32"/>
-      <c r="M113" s="14"/>
-      <c r="N113" s="32"/>
-      <c r="O113" s="32"/>
-      <c r="P113" s="32"/>
-      <c r="Q113" s="32"/>
-      <c r="R113" s="32"/>
-      <c r="S113" s="32"/>
-      <c r="T113" s="32"/>
-      <c r="U113" s="32"/>
-      <c r="V113" s="32"/>
-      <c r="W113" s="32"/>
-      <c r="X113" s="32"/>
-      <c r="Y113" s="32"/>
-      <c r="Z113" s="32"/>
-      <c r="AA113" s="32"/>
-      <c r="AB113" s="14"/>
-      <c r="AC113" s="14"/>
-      <c r="AD113" s="14"/>
-      <c r="AE113" s="14"/>
-      <c r="AF113" s="15"/>
+      <c r="D113" s="5"/>
+      <c r="E113" s="5"/>
+      <c r="F113" s="5"/>
+      <c r="G113" s="5"/>
+      <c r="H113" s="5"/>
+      <c r="I113" s="5"/>
+      <c r="J113" s="5"/>
+      <c r="K113" s="5"/>
+      <c r="M113" s="5"/>
+      <c r="AB113" s="5"/>
+      <c r="AC113" s="5"/>
+      <c r="AD113" s="5"/>
+      <c r="AE113" s="5"/>
+      <c r="AF113" s="6"/>
       <c r="AG113" s="6"/>
       <c r="AH113" s="6"/>
     </row>
     <row r="114" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="32"/>
-      <c r="B114" s="32"/>
-      <c r="C114" s="32"/>
-      <c r="D114" s="14"/>
-      <c r="E114" s="14"/>
-      <c r="F114" s="14"/>
-      <c r="G114" s="14"/>
-      <c r="H114" s="14"/>
-      <c r="I114" s="14"/>
-      <c r="J114" s="14"/>
-      <c r="K114" s="14"/>
-      <c r="L114" s="32"/>
-      <c r="M114" s="14"/>
-      <c r="N114" s="32"/>
-      <c r="O114" s="32"/>
-      <c r="P114" s="32"/>
-      <c r="Q114" s="32"/>
-      <c r="R114" s="32"/>
-      <c r="S114" s="32"/>
-      <c r="T114" s="32"/>
-      <c r="U114" s="32"/>
-      <c r="V114" s="32"/>
-      <c r="W114" s="32"/>
-      <c r="X114" s="32"/>
-      <c r="Y114" s="32"/>
-      <c r="Z114" s="32"/>
-      <c r="AA114" s="32"/>
-      <c r="AB114" s="14"/>
-      <c r="AC114" s="14"/>
-      <c r="AD114" s="14"/>
-      <c r="AE114" s="14"/>
-      <c r="AF114" s="15"/>
+      <c r="D114" s="5"/>
+      <c r="E114" s="5"/>
+      <c r="F114" s="5"/>
+      <c r="G114" s="5"/>
+      <c r="H114" s="5"/>
+      <c r="I114" s="5"/>
+      <c r="J114" s="5"/>
+      <c r="K114" s="5"/>
+      <c r="M114" s="5"/>
+      <c r="AB114" s="5"/>
+      <c r="AC114" s="5"/>
+      <c r="AD114" s="5"/>
+      <c r="AE114" s="5"/>
+      <c r="AF114" s="6"/>
       <c r="AG114" s="6"/>
       <c r="AH114" s="6"/>
     </row>
     <row r="115" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="32"/>
-      <c r="B115" s="32"/>
-      <c r="C115" s="32"/>
-      <c r="D115" s="14"/>
-      <c r="E115" s="14"/>
-      <c r="F115" s="14"/>
-      <c r="G115" s="14"/>
-      <c r="H115" s="14"/>
-      <c r="I115" s="14"/>
-      <c r="J115" s="14"/>
-      <c r="K115" s="14"/>
-      <c r="L115" s="32"/>
-      <c r="M115" s="14"/>
-      <c r="N115" s="32"/>
-      <c r="O115" s="32"/>
-      <c r="P115" s="32"/>
-      <c r="Q115" s="32"/>
-      <c r="R115" s="32"/>
-      <c r="S115" s="32"/>
-      <c r="T115" s="32"/>
-      <c r="U115" s="32"/>
-      <c r="V115" s="32"/>
-      <c r="W115" s="32"/>
-      <c r="X115" s="32"/>
-      <c r="Y115" s="32"/>
-      <c r="Z115" s="32"/>
-      <c r="AA115" s="32"/>
-      <c r="AB115" s="14"/>
-      <c r="AC115" s="14"/>
-      <c r="AD115" s="14"/>
-      <c r="AE115" s="14"/>
-      <c r="AF115" s="15"/>
+      <c r="D115" s="5"/>
+      <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
+      <c r="G115" s="5"/>
+      <c r="H115" s="5"/>
+      <c r="I115" s="5"/>
+      <c r="J115" s="5"/>
+      <c r="K115" s="5"/>
+      <c r="M115" s="5"/>
+      <c r="AB115" s="5"/>
+      <c r="AC115" s="5"/>
+      <c r="AD115" s="5"/>
+      <c r="AE115" s="5"/>
+      <c r="AF115" s="6"/>
       <c r="AG115" s="6"/>
       <c r="AH115" s="6"/>
     </row>
     <row r="116" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="32"/>
-      <c r="B116" s="32"/>
-      <c r="C116" s="32"/>
-      <c r="D116" s="14"/>
-      <c r="E116" s="14"/>
-      <c r="F116" s="14"/>
-      <c r="G116" s="14"/>
-      <c r="H116" s="14"/>
-      <c r="I116" s="14"/>
-      <c r="J116" s="14"/>
-      <c r="K116" s="14"/>
-      <c r="L116" s="32"/>
-      <c r="M116" s="14"/>
-      <c r="N116" s="32"/>
-      <c r="O116" s="32"/>
-      <c r="P116" s="32"/>
-      <c r="Q116" s="32"/>
-      <c r="R116" s="32"/>
-      <c r="S116" s="32"/>
-      <c r="T116" s="32"/>
-      <c r="U116" s="32"/>
-      <c r="V116" s="32"/>
-      <c r="W116" s="32"/>
-      <c r="X116" s="32"/>
-      <c r="Y116" s="32"/>
-      <c r="Z116" s="32"/>
-      <c r="AA116" s="32"/>
-      <c r="AB116" s="14"/>
-      <c r="AC116" s="14"/>
-      <c r="AD116" s="14"/>
-      <c r="AE116" s="14"/>
-      <c r="AF116" s="15"/>
+      <c r="D116" s="5"/>
+      <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
+      <c r="G116" s="5"/>
+      <c r="H116" s="5"/>
+      <c r="I116" s="5"/>
+      <c r="J116" s="5"/>
+      <c r="K116" s="5"/>
+      <c r="M116" s="5"/>
+      <c r="AB116" s="5"/>
+      <c r="AC116" s="5"/>
+      <c r="AD116" s="5"/>
+      <c r="AE116" s="5"/>
+      <c r="AF116" s="6"/>
       <c r="AG116" s="6"/>
       <c r="AH116" s="6"/>
     </row>
     <row r="117" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="32"/>
-      <c r="B117" s="32"/>
-      <c r="C117" s="32"/>
-      <c r="D117" s="14"/>
-      <c r="E117" s="14"/>
-      <c r="F117" s="14"/>
-      <c r="G117" s="14"/>
-      <c r="H117" s="14"/>
-      <c r="I117" s="14"/>
-      <c r="J117" s="14"/>
-      <c r="K117" s="14"/>
-      <c r="L117" s="32"/>
-      <c r="M117" s="14"/>
-      <c r="N117" s="32"/>
-      <c r="O117" s="32"/>
-      <c r="P117" s="32"/>
-      <c r="Q117" s="32"/>
-      <c r="R117" s="32"/>
-      <c r="S117" s="32"/>
-      <c r="T117" s="32"/>
-      <c r="U117" s="32"/>
-      <c r="V117" s="32"/>
-      <c r="W117" s="32"/>
-      <c r="X117" s="32"/>
-      <c r="Y117" s="32"/>
-      <c r="Z117" s="32"/>
-      <c r="AA117" s="32"/>
-      <c r="AB117" s="14"/>
-      <c r="AC117" s="14"/>
-      <c r="AD117" s="14"/>
-      <c r="AE117" s="14"/>
-      <c r="AF117" s="15"/>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5"/>
+      <c r="H117" s="5"/>
+      <c r="I117" s="5"/>
+      <c r="J117" s="5"/>
+      <c r="K117" s="5"/>
+      <c r="M117" s="5"/>
+      <c r="AB117" s="5"/>
+      <c r="AC117" s="5"/>
+      <c r="AD117" s="5"/>
+      <c r="AE117" s="5"/>
+      <c r="AF117" s="6"/>
       <c r="AG117" s="6"/>
       <c r="AH117" s="6"/>
     </row>
     <row r="118" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="32"/>
-      <c r="B118" s="32"/>
-      <c r="C118" s="32"/>
-      <c r="D118" s="14"/>
-      <c r="E118" s="14"/>
-      <c r="F118" s="14"/>
-      <c r="G118" s="14"/>
-      <c r="H118" s="14"/>
-      <c r="I118" s="14"/>
-      <c r="J118" s="14"/>
-      <c r="K118" s="14"/>
-      <c r="L118" s="32"/>
-      <c r="M118" s="14"/>
-      <c r="N118" s="32"/>
-      <c r="O118" s="32"/>
-      <c r="P118" s="32"/>
-      <c r="Q118" s="32"/>
-      <c r="R118" s="32"/>
-      <c r="S118" s="32"/>
-      <c r="T118" s="32"/>
-      <c r="U118" s="32"/>
-      <c r="V118" s="32"/>
-      <c r="W118" s="32"/>
-      <c r="X118" s="32"/>
-      <c r="Y118" s="32"/>
-      <c r="Z118" s="32"/>
-      <c r="AA118" s="32"/>
-      <c r="AB118" s="14"/>
-      <c r="AC118" s="14"/>
-      <c r="AD118" s="14"/>
-      <c r="AE118" s="14"/>
-      <c r="AF118" s="15"/>
+      <c r="D118" s="5"/>
+      <c r="E118" s="5"/>
+      <c r="F118" s="5"/>
+      <c r="G118" s="5"/>
+      <c r="H118" s="5"/>
+      <c r="I118" s="5"/>
+      <c r="J118" s="5"/>
+      <c r="K118" s="5"/>
+      <c r="M118" s="5"/>
+      <c r="AB118" s="5"/>
+      <c r="AC118" s="5"/>
+      <c r="AD118" s="5"/>
+      <c r="AE118" s="5"/>
+      <c r="AF118" s="6"/>
       <c r="AG118" s="6"/>
       <c r="AH118" s="6"/>
     </row>
     <row r="119" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="32"/>
-      <c r="B119" s="32"/>
-      <c r="C119" s="32"/>
-      <c r="D119" s="14"/>
-      <c r="E119" s="14"/>
-      <c r="F119" s="14"/>
-      <c r="G119" s="14"/>
-      <c r="H119" s="14"/>
-      <c r="I119" s="14"/>
-      <c r="J119" s="14"/>
-      <c r="K119" s="14"/>
-      <c r="L119" s="32"/>
-      <c r="M119" s="14"/>
-      <c r="N119" s="32"/>
-      <c r="O119" s="32"/>
-      <c r="P119" s="32"/>
-      <c r="Q119" s="32"/>
-      <c r="R119" s="32"/>
-      <c r="S119" s="32"/>
-      <c r="T119" s="32"/>
-      <c r="U119" s="32"/>
-      <c r="V119" s="32"/>
-      <c r="W119" s="32"/>
-      <c r="X119" s="32"/>
-      <c r="Y119" s="32"/>
-      <c r="Z119" s="32"/>
-      <c r="AA119" s="32"/>
-      <c r="AB119" s="14"/>
-      <c r="AC119" s="14"/>
-      <c r="AD119" s="14"/>
-      <c r="AE119" s="14"/>
-      <c r="AF119" s="15"/>
+      <c r="D119" s="5"/>
+      <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
+      <c r="G119" s="5"/>
+      <c r="H119" s="5"/>
+      <c r="I119" s="5"/>
+      <c r="J119" s="5"/>
+      <c r="K119" s="5"/>
+      <c r="M119" s="5"/>
+      <c r="AB119" s="5"/>
+      <c r="AC119" s="5"/>
+      <c r="AD119" s="5"/>
+      <c r="AE119" s="5"/>
+      <c r="AF119" s="6"/>
       <c r="AG119" s="6"/>
       <c r="AH119" s="6"/>
     </row>
     <row r="120" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="32"/>
-      <c r="B120" s="32"/>
-      <c r="C120" s="32"/>
-      <c r="D120" s="14"/>
-      <c r="E120" s="14"/>
-      <c r="F120" s="14"/>
-      <c r="G120" s="14"/>
-      <c r="H120" s="14"/>
-      <c r="I120" s="14"/>
-      <c r="J120" s="14"/>
-      <c r="K120" s="14"/>
-      <c r="L120" s="32"/>
-      <c r="M120" s="14"/>
-      <c r="N120" s="32"/>
-      <c r="O120" s="32"/>
-      <c r="P120" s="32"/>
-      <c r="Q120" s="32"/>
-      <c r="R120" s="32"/>
-      <c r="S120" s="32"/>
-      <c r="T120" s="32"/>
-      <c r="U120" s="32"/>
-      <c r="V120" s="32"/>
-      <c r="W120" s="32"/>
-      <c r="X120" s="32"/>
-      <c r="Y120" s="32"/>
-      <c r="Z120" s="32"/>
-      <c r="AA120" s="32"/>
-      <c r="AB120" s="14"/>
-      <c r="AC120" s="14"/>
-      <c r="AD120" s="14"/>
-      <c r="AE120" s="14"/>
-      <c r="AF120" s="15"/>
+      <c r="D120" s="5"/>
+      <c r="E120" s="5"/>
+      <c r="F120" s="5"/>
+      <c r="G120" s="5"/>
+      <c r="H120" s="5"/>
+      <c r="I120" s="5"/>
+      <c r="J120" s="5"/>
+      <c r="K120" s="5"/>
+      <c r="M120" s="5"/>
+      <c r="AB120" s="5"/>
+      <c r="AC120" s="5"/>
+      <c r="AD120" s="5"/>
+      <c r="AE120" s="5"/>
+      <c r="AF120" s="6"/>
       <c r="AG120" s="6"/>
       <c r="AH120" s="6"/>
     </row>
     <row r="121" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="32"/>
-      <c r="B121" s="32"/>
-      <c r="C121" s="32"/>
-      <c r="D121" s="14"/>
-      <c r="E121" s="14"/>
-      <c r="F121" s="14"/>
-      <c r="G121" s="14"/>
-      <c r="H121" s="14"/>
-      <c r="I121" s="14"/>
-      <c r="J121" s="14"/>
-      <c r="K121" s="14"/>
-      <c r="L121" s="14"/>
-      <c r="M121" s="14"/>
-      <c r="N121" s="32"/>
-      <c r="O121" s="32"/>
-      <c r="P121" s="32"/>
-      <c r="Q121" s="32"/>
-      <c r="R121" s="32"/>
-      <c r="S121" s="32"/>
-      <c r="T121" s="32"/>
-      <c r="U121" s="32"/>
-      <c r="V121" s="32"/>
-      <c r="W121" s="32"/>
-      <c r="X121" s="32"/>
-      <c r="Y121" s="32"/>
-      <c r="Z121" s="32"/>
-      <c r="AA121" s="32"/>
-      <c r="AB121" s="14"/>
-      <c r="AC121" s="14"/>
-      <c r="AD121" s="14"/>
-      <c r="AE121" s="14"/>
-      <c r="AF121" s="15"/>
+      <c r="D121" s="5"/>
+      <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
+      <c r="G121" s="5"/>
+      <c r="H121" s="5"/>
+      <c r="I121" s="5"/>
+      <c r="J121" s="5"/>
+      <c r="K121" s="5"/>
+      <c r="L121" s="5"/>
+      <c r="M121" s="5"/>
+      <c r="AB121" s="5"/>
+      <c r="AC121" s="5"/>
+      <c r="AD121" s="5"/>
+      <c r="AE121" s="5"/>
+      <c r="AF121" s="6"/>
       <c r="AG121" s="6"/>
       <c r="AH121" s="6"/>
     </row>
     <row r="122" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="14"/>
-      <c r="B122" s="14"/>
-      <c r="C122" s="14"/>
-      <c r="D122" s="14"/>
-      <c r="E122" s="14"/>
-      <c r="F122" s="14"/>
-      <c r="G122" s="14"/>
-      <c r="H122" s="14"/>
-      <c r="I122" s="14"/>
-      <c r="J122" s="14"/>
-      <c r="K122" s="14"/>
-      <c r="L122" s="14"/>
-      <c r="M122" s="14"/>
-      <c r="N122" s="14"/>
-      <c r="O122" s="14"/>
-      <c r="P122" s="14"/>
-      <c r="Q122" s="14"/>
-      <c r="R122" s="14"/>
-      <c r="S122" s="14"/>
-      <c r="T122" s="14"/>
-      <c r="U122" s="14"/>
-      <c r="V122" s="14"/>
-      <c r="W122" s="14"/>
-      <c r="X122" s="14"/>
-      <c r="Y122" s="14"/>
-      <c r="Z122" s="14"/>
-      <c r="AA122" s="14"/>
-      <c r="AB122" s="14"/>
-      <c r="AC122" s="14"/>
-      <c r="AD122" s="14"/>
-      <c r="AE122" s="14"/>
-      <c r="AF122" s="15"/>
+      <c r="A122" s="5"/>
+      <c r="B122" s="5"/>
+      <c r="C122" s="5"/>
+      <c r="D122" s="5"/>
+      <c r="E122" s="5"/>
+      <c r="F122" s="5"/>
+      <c r="G122" s="5"/>
+      <c r="H122" s="5"/>
+      <c r="I122" s="5"/>
+      <c r="J122" s="5"/>
+      <c r="K122" s="5"/>
+      <c r="L122" s="5"/>
+      <c r="M122" s="5"/>
+      <c r="N122" s="5"/>
+      <c r="O122" s="5"/>
+      <c r="P122" s="5"/>
+      <c r="Q122" s="5"/>
+      <c r="R122" s="5"/>
+      <c r="S122" s="5"/>
+      <c r="T122" s="5"/>
+      <c r="U122" s="5"/>
+      <c r="V122" s="5"/>
+      <c r="W122" s="5"/>
+      <c r="X122" s="5"/>
+      <c r="Y122" s="5"/>
+      <c r="Z122" s="5"/>
+      <c r="AA122" s="5"/>
+      <c r="AB122" s="5"/>
+      <c r="AC122" s="5"/>
+      <c r="AD122" s="5"/>
+      <c r="AE122" s="5"/>
+      <c r="AF122" s="6"/>
       <c r="AG122" s="6"/>
       <c r="AH122" s="6"/>
     </row>

</xml_diff>